<commit_message>
chore: init repo & add CheckerUI_win.spec
</commit_message>
<xml_diff>
--- a/L2++_组合票.xlsx
+++ b/L2++_组合票.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10720"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhongwenjie/程序/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D69C1E-8EC1-E84A-A497-0B3E85922048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="作业组合票" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="29">
   <si>
     <t>连续投入L2++等待时间</t>
   </si>
@@ -94,39 +88,30 @@
     <t>37.5</t>
   </si>
   <si>
-    <t>入站等待0秒；总等待75秒</t>
+    <t>入站等待7.5秒；总等待75秒</t>
   </si>
   <si>
-    <t>等待5.5秒（电检准备 → 电检1）</t>
+    <t>7.5</t>
   </si>
   <si>
-    <t>5.5</t>
+    <t>等待67.5秒（电检1 → 电检2）</t>
   </si>
   <si>
-    <t>等待69.5秒（电检1 → 电检2）</t>
+    <t>67.5</t>
   </si>
   <si>
-    <t>69.5</t>
-  </si>
-  <si>
-    <t>入站等待0秒；总等待112.5秒</t>
-  </si>
-  <si>
-    <t>等待43秒（电检准备 → 电检1）</t>
-  </si>
-  <si>
-    <t>43</t>
+    <t>入站等待37.5秒；总等待105秒</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -134,19 +119,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -167,6 +145,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF9C27B0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9800"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3F51B5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF009688"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -179,31 +175,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF9800"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF795548"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF2196F3"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF3F51B5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF8BC34A"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -247,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -267,32 +239,23 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -330,7 +293,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -364,7 +327,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -399,10 +361,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -575,15 +536,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AGF45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AGF43"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="36.6640625" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="864" width="3.5" customWidth="1"/>
+    <col min="1" max="1" width="36.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="864" width="3.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:864">
@@ -3623,26 +3584,26 @@
       <c r="D9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="NB9" s="10"/>
-      <c r="NC9" s="10"/>
-      <c r="ND9" s="10"/>
-      <c r="NE9" s="10"/>
-      <c r="NF9" s="10"/>
-      <c r="NG9" s="10"/>
-      <c r="NH9" s="10"/>
-      <c r="NI9" s="10"/>
-      <c r="NJ9" s="10"/>
-      <c r="NK9" s="10"/>
-      <c r="NL9" s="10"/>
-      <c r="NM9" s="10"/>
-      <c r="NN9" s="10"/>
-      <c r="NO9" s="10"/>
-      <c r="NP9" s="10"/>
-      <c r="NQ9" s="10"/>
-      <c r="NR9" s="10"/>
-      <c r="NS9" s="10"/>
-      <c r="NT9" s="10"/>
-      <c r="NU9" s="10"/>
+      <c r="NB9" s="5"/>
+      <c r="NC9" s="5"/>
+      <c r="ND9" s="5"/>
+      <c r="NE9" s="5"/>
+      <c r="NF9" s="5"/>
+      <c r="NG9" s="5"/>
+      <c r="NH9" s="5"/>
+      <c r="NI9" s="5"/>
+      <c r="NJ9" s="5"/>
+      <c r="NK9" s="5"/>
+      <c r="NL9" s="5"/>
+      <c r="NM9" s="5"/>
+      <c r="NN9" s="5"/>
+      <c r="NO9" s="5"/>
+      <c r="NP9" s="5"/>
+      <c r="NQ9" s="5"/>
+      <c r="NR9" s="5"/>
+      <c r="NS9" s="5"/>
+      <c r="NT9" s="5"/>
+      <c r="NU9" s="5"/>
     </row>
     <row r="10" spans="1:864">
       <c r="A10" s="2"/>
@@ -3653,36 +3614,36 @@
       <c r="D10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="NV10" s="11"/>
-      <c r="NW10" s="11"/>
-      <c r="NX10" s="11"/>
-      <c r="NY10" s="11"/>
-      <c r="NZ10" s="11"/>
-      <c r="OA10" s="11"/>
-      <c r="OB10" s="11"/>
-      <c r="OC10" s="11"/>
-      <c r="OD10" s="11"/>
-      <c r="OE10" s="11"/>
-      <c r="OF10" s="11"/>
-      <c r="OG10" s="11"/>
-      <c r="OH10" s="11"/>
-      <c r="OI10" s="11"/>
-      <c r="OJ10" s="11"/>
-      <c r="OK10" s="11"/>
-      <c r="OL10" s="11"/>
-      <c r="OM10" s="11"/>
-      <c r="ON10" s="11"/>
-      <c r="OO10" s="11"/>
-      <c r="OP10" s="11"/>
-      <c r="OQ10" s="11"/>
-      <c r="OR10" s="11"/>
-      <c r="OS10" s="11"/>
-      <c r="OT10" s="11"/>
-      <c r="OU10" s="11"/>
-      <c r="OV10" s="11"/>
-      <c r="OW10" s="11"/>
-      <c r="OX10" s="11"/>
-      <c r="OY10" s="11"/>
+      <c r="NV10" s="10"/>
+      <c r="NW10" s="10"/>
+      <c r="NX10" s="10"/>
+      <c r="NY10" s="10"/>
+      <c r="NZ10" s="10"/>
+      <c r="OA10" s="10"/>
+      <c r="OB10" s="10"/>
+      <c r="OC10" s="10"/>
+      <c r="OD10" s="10"/>
+      <c r="OE10" s="10"/>
+      <c r="OF10" s="10"/>
+      <c r="OG10" s="10"/>
+      <c r="OH10" s="10"/>
+      <c r="OI10" s="10"/>
+      <c r="OJ10" s="10"/>
+      <c r="OK10" s="10"/>
+      <c r="OL10" s="10"/>
+      <c r="OM10" s="10"/>
+      <c r="ON10" s="10"/>
+      <c r="OO10" s="10"/>
+      <c r="OP10" s="10"/>
+      <c r="OQ10" s="10"/>
+      <c r="OR10" s="10"/>
+      <c r="OS10" s="10"/>
+      <c r="OT10" s="10"/>
+      <c r="OU10" s="10"/>
+      <c r="OV10" s="10"/>
+      <c r="OW10" s="10"/>
+      <c r="OX10" s="10"/>
+      <c r="OY10" s="10"/>
     </row>
     <row r="12" spans="1:864">
       <c r="A12" s="2" t="s">
@@ -3958,54 +3919,54 @@
       <c r="MJ15" s="7"/>
     </row>
     <row r="16" spans="1:864">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>22</v>
       </c>
       <c r="B16" s="4"/>
-      <c r="C16" s="12"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="MJ16" s="13"/>
-      <c r="MK16" s="13"/>
-      <c r="ML16" s="13"/>
-      <c r="MM16" s="13"/>
-      <c r="MN16" s="13"/>
-      <c r="MO16" s="13"/>
-      <c r="MP16" s="13"/>
-      <c r="MQ16" s="13"/>
-      <c r="MR16" s="13"/>
-      <c r="MS16" s="13"/>
-      <c r="MT16" s="13"/>
-      <c r="MU16" s="13"/>
-      <c r="MV16" s="13"/>
-      <c r="MW16" s="13"/>
-      <c r="MX16" s="13"/>
-      <c r="MY16" s="13"/>
-      <c r="MZ16" s="13"/>
-      <c r="NA16" s="13"/>
-      <c r="NB16" s="13"/>
-      <c r="NC16" s="13"/>
-      <c r="ND16" s="13"/>
-      <c r="NE16" s="13"/>
-      <c r="NF16" s="13"/>
-      <c r="NG16" s="13"/>
-      <c r="NH16" s="13"/>
-      <c r="NI16" s="13"/>
-      <c r="NJ16" s="13"/>
-      <c r="NK16" s="13"/>
-      <c r="NL16" s="13"/>
-      <c r="NM16" s="13"/>
-      <c r="NN16" s="13"/>
-      <c r="NO16" s="13"/>
-      <c r="NP16" s="13"/>
-      <c r="NQ16" s="13"/>
-      <c r="NR16" s="13"/>
-      <c r="NS16" s="13"/>
-      <c r="NT16" s="13"/>
-      <c r="NU16" s="13"/>
+      <c r="MJ16" s="12"/>
+      <c r="MK16" s="12"/>
+      <c r="ML16" s="12"/>
+      <c r="MM16" s="12"/>
+      <c r="MN16" s="12"/>
+      <c r="MO16" s="12"/>
+      <c r="MP16" s="12"/>
+      <c r="MQ16" s="12"/>
+      <c r="MR16" s="12"/>
+      <c r="MS16" s="12"/>
+      <c r="MT16" s="12"/>
+      <c r="MU16" s="12"/>
+      <c r="MV16" s="12"/>
+      <c r="MW16" s="12"/>
+      <c r="MX16" s="12"/>
+      <c r="MY16" s="12"/>
+      <c r="MZ16" s="12"/>
+      <c r="NA16" s="12"/>
+      <c r="NB16" s="12"/>
+      <c r="NC16" s="12"/>
+      <c r="ND16" s="12"/>
+      <c r="NE16" s="12"/>
+      <c r="NF16" s="12"/>
+      <c r="NG16" s="12"/>
+      <c r="NH16" s="12"/>
+      <c r="NI16" s="12"/>
+      <c r="NJ16" s="12"/>
+      <c r="NK16" s="12"/>
+      <c r="NL16" s="12"/>
+      <c r="NM16" s="12"/>
+      <c r="NN16" s="12"/>
+      <c r="NO16" s="12"/>
+      <c r="NP16" s="12"/>
+      <c r="NQ16" s="12"/>
+      <c r="NR16" s="12"/>
+      <c r="NS16" s="12"/>
+      <c r="NT16" s="12"/>
+      <c r="NU16" s="12"/>
     </row>
-    <row r="17" spans="1:684">
+    <row r="17" spans="1:714">
       <c r="A17" s="2"/>
       <c r="B17" s="4"/>
       <c r="C17" s="2" t="s">
@@ -4085,7 +4046,7 @@
       <c r="QL17" s="7"/>
       <c r="QM17" s="7"/>
     </row>
-    <row r="18" spans="1:684">
+    <row r="18" spans="1:714">
       <c r="A18" s="2"/>
       <c r="B18" s="4"/>
       <c r="C18" s="2" t="s">
@@ -4125,7 +4086,7 @@
       <c r="RP18" s="8"/>
       <c r="RQ18" s="8"/>
     </row>
-    <row r="19" spans="1:684">
+    <row r="19" spans="1:714">
       <c r="A19" s="2"/>
       <c r="B19" s="4"/>
       <c r="C19" s="2" t="s">
@@ -4166,7 +4127,7 @@
       <c r="ST19" s="9"/>
       <c r="SU19" s="9"/>
     </row>
-    <row r="20" spans="1:684">
+    <row r="20" spans="1:714">
       <c r="A20" s="2"/>
       <c r="B20" s="4"/>
       <c r="C20" s="2" t="s">
@@ -4175,29 +4136,29 @@
       <c r="D20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="SU20" s="10"/>
-      <c r="SV20" s="10"/>
-      <c r="SW20" s="10"/>
-      <c r="SX20" s="10"/>
-      <c r="SY20" s="10"/>
-      <c r="SZ20" s="10"/>
-      <c r="TA20" s="10"/>
-      <c r="TB20" s="10"/>
-      <c r="TC20" s="10"/>
-      <c r="TD20" s="10"/>
-      <c r="TE20" s="10"/>
-      <c r="TF20" s="10"/>
-      <c r="TG20" s="10"/>
-      <c r="TH20" s="10"/>
-      <c r="TI20" s="10"/>
-      <c r="TJ20" s="10"/>
-      <c r="TK20" s="10"/>
-      <c r="TL20" s="10"/>
-      <c r="TM20" s="10"/>
-      <c r="TN20" s="10"/>
-      <c r="TO20" s="10"/>
+      <c r="SU20" s="5"/>
+      <c r="SV20" s="5"/>
+      <c r="SW20" s="5"/>
+      <c r="SX20" s="5"/>
+      <c r="SY20" s="5"/>
+      <c r="SZ20" s="5"/>
+      <c r="TA20" s="5"/>
+      <c r="TB20" s="5"/>
+      <c r="TC20" s="5"/>
+      <c r="TD20" s="5"/>
+      <c r="TE20" s="5"/>
+      <c r="TF20" s="5"/>
+      <c r="TG20" s="5"/>
+      <c r="TH20" s="5"/>
+      <c r="TI20" s="5"/>
+      <c r="TJ20" s="5"/>
+      <c r="TK20" s="5"/>
+      <c r="TL20" s="5"/>
+      <c r="TM20" s="5"/>
+      <c r="TN20" s="5"/>
+      <c r="TO20" s="5"/>
     </row>
-    <row r="21" spans="1:684">
+    <row r="21" spans="1:714">
       <c r="A21" s="2"/>
       <c r="B21" s="4"/>
       <c r="C21" s="2" t="s">
@@ -4206,49 +4167,283 @@
       <c r="D21" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="TO21" s="11"/>
-      <c r="TP21" s="11"/>
-      <c r="TQ21" s="11"/>
-      <c r="TR21" s="11"/>
-      <c r="TS21" s="11"/>
-      <c r="TT21" s="11"/>
-      <c r="TU21" s="11"/>
-      <c r="TV21" s="11"/>
-      <c r="TW21" s="11"/>
-      <c r="TX21" s="11"/>
-      <c r="TY21" s="11"/>
-      <c r="TZ21" s="11"/>
-      <c r="UA21" s="11"/>
-      <c r="UB21" s="11"/>
-      <c r="UC21" s="11"/>
-      <c r="UD21" s="11"/>
-      <c r="UE21" s="11"/>
-      <c r="UF21" s="11"/>
-      <c r="UG21" s="11"/>
-      <c r="UH21" s="11"/>
-      <c r="UI21" s="11"/>
-      <c r="UJ21" s="11"/>
-      <c r="UK21" s="11"/>
-      <c r="UL21" s="11"/>
-      <c r="UM21" s="11"/>
-      <c r="UN21" s="11"/>
-      <c r="UO21" s="11"/>
-      <c r="UP21" s="11"/>
-      <c r="UQ21" s="11"/>
-      <c r="UR21" s="11"/>
-      <c r="US21" s="11"/>
+      <c r="TO21" s="10"/>
+      <c r="TP21" s="10"/>
+      <c r="TQ21" s="10"/>
+      <c r="TR21" s="10"/>
+      <c r="TS21" s="10"/>
+      <c r="TT21" s="10"/>
+      <c r="TU21" s="10"/>
+      <c r="TV21" s="10"/>
+      <c r="TW21" s="10"/>
+      <c r="TX21" s="10"/>
+      <c r="TY21" s="10"/>
+      <c r="TZ21" s="10"/>
+      <c r="UA21" s="10"/>
+      <c r="UB21" s="10"/>
+      <c r="UC21" s="10"/>
+      <c r="UD21" s="10"/>
+      <c r="UE21" s="10"/>
+      <c r="UF21" s="10"/>
+      <c r="UG21" s="10"/>
+      <c r="UH21" s="10"/>
+      <c r="UI21" s="10"/>
+      <c r="UJ21" s="10"/>
+      <c r="UK21" s="10"/>
+      <c r="UL21" s="10"/>
+      <c r="UM21" s="10"/>
+      <c r="UN21" s="10"/>
+      <c r="UO21" s="10"/>
+      <c r="UP21" s="10"/>
+      <c r="UQ21" s="10"/>
+      <c r="UR21" s="10"/>
+      <c r="US21" s="10"/>
     </row>
-    <row r="23" spans="1:684">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:714">
+      <c r="A23" s="11" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="3">
         <v>3</v>
       </c>
       <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="D23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="12"/>
+      <c r="Q23" s="12"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="12"/>
+      <c r="T23" s="12"/>
+      <c r="U23" s="12"/>
+      <c r="V23" s="12"/>
+      <c r="W23" s="12"/>
+      <c r="X23" s="12"/>
+      <c r="Y23" s="12"/>
+      <c r="Z23" s="12"/>
+      <c r="AA23" s="12"/>
+      <c r="AB23" s="12"/>
+      <c r="AC23" s="12"/>
+      <c r="AD23" s="12"/>
+      <c r="AE23" s="12"/>
+      <c r="AF23" s="12"/>
+      <c r="AG23" s="12"/>
+      <c r="AH23" s="12"/>
+      <c r="AI23" s="12"/>
+      <c r="AJ23" s="12"/>
+      <c r="AK23" s="12"/>
+      <c r="AL23" s="12"/>
+      <c r="AM23" s="12"/>
+      <c r="AN23" s="12"/>
+      <c r="AO23" s="12"/>
+      <c r="AP23" s="12"/>
+      <c r="AQ23" s="12"/>
+      <c r="AR23" s="12"/>
+      <c r="AS23" s="12"/>
+      <c r="AT23" s="12"/>
+      <c r="AU23" s="12"/>
+      <c r="AV23" s="12"/>
+      <c r="AW23" s="12"/>
+      <c r="AX23" s="12"/>
+      <c r="AY23" s="12"/>
+      <c r="AZ23" s="12"/>
+      <c r="BA23" s="12"/>
+      <c r="BB23" s="12"/>
+      <c r="BC23" s="12"/>
+      <c r="BD23" s="12"/>
+      <c r="BE23" s="12"/>
+      <c r="BF23" s="12"/>
+      <c r="BG23" s="12"/>
+      <c r="BH23" s="12"/>
+      <c r="BI23" s="12"/>
+      <c r="BJ23" s="12"/>
+      <c r="BK23" s="12"/>
+      <c r="BL23" s="12"/>
+      <c r="BM23" s="12"/>
+      <c r="BN23" s="12"/>
+      <c r="BO23" s="12"/>
+      <c r="BP23" s="12"/>
+      <c r="BQ23" s="12"/>
+      <c r="BR23" s="12"/>
+      <c r="BS23" s="12"/>
+      <c r="BT23" s="12"/>
+      <c r="BU23" s="12"/>
+      <c r="BV23" s="12"/>
+      <c r="BW23" s="12"/>
+      <c r="BX23" s="12"/>
+      <c r="BY23" s="12"/>
+      <c r="BZ23" s="12"/>
+      <c r="CA23" s="12"/>
+      <c r="CB23" s="12"/>
+      <c r="CC23" s="12"/>
+      <c r="CD23" s="12"/>
+      <c r="CE23" s="12"/>
+      <c r="CF23" s="12"/>
+      <c r="CG23" s="12"/>
+      <c r="CH23" s="12"/>
+      <c r="CI23" s="12"/>
+      <c r="CJ23" s="12"/>
+      <c r="CK23" s="12"/>
+      <c r="CL23" s="12"/>
+      <c r="CM23" s="12"/>
+      <c r="CN23" s="12"/>
+      <c r="CO23" s="12"/>
+      <c r="CP23" s="12"/>
+      <c r="CQ23" s="12"/>
+      <c r="CR23" s="12"/>
+      <c r="CS23" s="12"/>
+      <c r="CT23" s="12"/>
+      <c r="CU23" s="12"/>
+      <c r="CV23" s="12"/>
+      <c r="CW23" s="12"/>
+      <c r="CX23" s="12"/>
+      <c r="CY23" s="12"/>
+      <c r="CZ23" s="12"/>
+      <c r="DA23" s="12"/>
+      <c r="DB23" s="12"/>
+      <c r="DC23" s="12"/>
+      <c r="DD23" s="12"/>
+      <c r="DE23" s="12"/>
+      <c r="DF23" s="12"/>
+      <c r="DG23" s="12"/>
+      <c r="DH23" s="12"/>
+      <c r="DI23" s="12"/>
+      <c r="DJ23" s="12"/>
+      <c r="DK23" s="12"/>
+      <c r="DL23" s="12"/>
+      <c r="DM23" s="12"/>
+      <c r="DN23" s="12"/>
+      <c r="DO23" s="12"/>
+      <c r="DP23" s="12"/>
+      <c r="DQ23" s="12"/>
+      <c r="DR23" s="12"/>
+      <c r="DS23" s="12"/>
+      <c r="DT23" s="12"/>
+      <c r="DU23" s="12"/>
+      <c r="DV23" s="12"/>
+      <c r="DW23" s="12"/>
+      <c r="DX23" s="12"/>
+      <c r="DY23" s="12"/>
+      <c r="DZ23" s="12"/>
+      <c r="EA23" s="12"/>
+      <c r="EB23" s="12"/>
+      <c r="EC23" s="12"/>
+      <c r="ED23" s="12"/>
+      <c r="EE23" s="12"/>
+      <c r="EF23" s="12"/>
+      <c r="EG23" s="12"/>
+      <c r="EH23" s="12"/>
+      <c r="EI23" s="12"/>
+      <c r="EJ23" s="12"/>
+      <c r="EK23" s="12"/>
+      <c r="EL23" s="12"/>
+      <c r="EM23" s="12"/>
+      <c r="EN23" s="12"/>
+      <c r="EO23" s="12"/>
+      <c r="EP23" s="12"/>
+      <c r="EQ23" s="12"/>
+      <c r="ER23" s="12"/>
+      <c r="ES23" s="12"/>
+      <c r="ET23" s="12"/>
+      <c r="EU23" s="12"/>
+      <c r="EV23" s="12"/>
+      <c r="EW23" s="12"/>
+      <c r="EX23" s="12"/>
+      <c r="EY23" s="12"/>
+      <c r="EZ23" s="12"/>
+      <c r="FA23" s="12"/>
+      <c r="FB23" s="12"/>
+      <c r="FC23" s="12"/>
+      <c r="FD23" s="12"/>
+      <c r="FE23" s="12"/>
+      <c r="FF23" s="12"/>
+      <c r="FG23" s="12"/>
+      <c r="FH23" s="12"/>
+      <c r="FI23" s="12"/>
+      <c r="FJ23" s="12"/>
+      <c r="FK23" s="12"/>
+      <c r="FL23" s="12"/>
+      <c r="FM23" s="12"/>
+      <c r="FN23" s="12"/>
+      <c r="FO23" s="12"/>
+      <c r="FP23" s="12"/>
+      <c r="FQ23" s="12"/>
+      <c r="FR23" s="12"/>
+      <c r="FS23" s="12"/>
+      <c r="FT23" s="12"/>
+      <c r="FU23" s="12"/>
+      <c r="FV23" s="12"/>
+      <c r="FW23" s="12"/>
+      <c r="FX23" s="12"/>
+      <c r="FY23" s="12"/>
+      <c r="FZ23" s="12"/>
+      <c r="GA23" s="12"/>
+      <c r="GB23" s="12"/>
+      <c r="GC23" s="12"/>
+      <c r="GD23" s="12"/>
+      <c r="GE23" s="12"/>
+      <c r="GF23" s="12"/>
+      <c r="GG23" s="12"/>
+      <c r="GH23" s="12"/>
+      <c r="GI23" s="12"/>
+      <c r="GJ23" s="12"/>
+      <c r="GK23" s="12"/>
+      <c r="GL23" s="12"/>
+      <c r="GM23" s="12"/>
+      <c r="GN23" s="12"/>
+      <c r="GO23" s="12"/>
+      <c r="GP23" s="12"/>
+      <c r="GQ23" s="12"/>
+      <c r="GR23" s="12"/>
+      <c r="GS23" s="12"/>
+      <c r="GT23" s="12"/>
+      <c r="GU23" s="12"/>
+      <c r="GV23" s="12"/>
+      <c r="GW23" s="12"/>
+      <c r="GX23" s="12"/>
+      <c r="GY23" s="12"/>
+      <c r="GZ23" s="12"/>
+      <c r="HA23" s="12"/>
+      <c r="HB23" s="12"/>
+      <c r="HC23" s="12"/>
+      <c r="HD23" s="12"/>
+      <c r="HE23" s="12"/>
+      <c r="HF23" s="12"/>
+      <c r="HG23" s="12"/>
+      <c r="HH23" s="12"/>
+      <c r="HI23" s="12"/>
+      <c r="HJ23" s="12"/>
+      <c r="HK23" s="12"/>
+      <c r="HL23" s="12"/>
+      <c r="HM23" s="12"/>
+      <c r="HN23" s="12"/>
+      <c r="HO23" s="12"/>
+      <c r="HP23" s="12"/>
+      <c r="HQ23" s="12"/>
+      <c r="HR23" s="12"/>
+      <c r="HS23" s="12"/>
+      <c r="HT23" s="12"/>
+      <c r="HU23" s="12"/>
+      <c r="HV23" s="12"/>
+      <c r="HW23" s="12"/>
+      <c r="HX23" s="12"/>
+      <c r="HY23" s="12"/>
+      <c r="HZ23" s="12"/>
+      <c r="IA23" s="12"/>
+      <c r="IB23" s="12"/>
     </row>
-    <row r="24" spans="1:684">
+    <row r="24" spans="1:714">
       <c r="A24" s="2"/>
       <c r="B24" s="4"/>
       <c r="C24" s="2" t="s">
@@ -4257,13 +4452,6 @@
       <c r="D24" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="HU24" s="5"/>
-      <c r="HV24" s="5"/>
-      <c r="HW24" s="5"/>
-      <c r="HX24" s="5"/>
-      <c r="HY24" s="5"/>
-      <c r="HZ24" s="5"/>
-      <c r="IA24" s="5"/>
       <c r="IB24" s="5"/>
       <c r="IC24" s="5"/>
       <c r="ID24" s="5"/>
@@ -4369,8 +4557,16 @@
       <c r="LZ24" s="5"/>
       <c r="MA24" s="5"/>
       <c r="MB24" s="5"/>
+      <c r="MC24" s="5"/>
+      <c r="MD24" s="5"/>
+      <c r="ME24" s="5"/>
+      <c r="MF24" s="5"/>
+      <c r="MG24" s="5"/>
+      <c r="MH24" s="5"/>
+      <c r="MI24" s="5"/>
+      <c r="MJ24" s="5"/>
     </row>
-    <row r="25" spans="1:684">
+    <row r="25" spans="1:714">
       <c r="A25" s="2"/>
       <c r="B25" s="4"/>
       <c r="C25" s="2" t="s">
@@ -4379,13 +4575,6 @@
       <c r="D25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="MC25" s="6"/>
-      <c r="MD25" s="6"/>
-      <c r="ME25" s="6"/>
-      <c r="MF25" s="6"/>
-      <c r="MG25" s="6"/>
-      <c r="MH25" s="6"/>
-      <c r="MI25" s="6"/>
       <c r="MJ25" s="6"/>
       <c r="MK25" s="6"/>
       <c r="ML25" s="6"/>
@@ -4419,1066 +4608,1381 @@
       <c r="NN25" s="6"/>
       <c r="NO25" s="6"/>
       <c r="NP25" s="6"/>
+      <c r="NQ25" s="6"/>
+      <c r="NR25" s="6"/>
+      <c r="NS25" s="6"/>
+      <c r="NT25" s="6"/>
+      <c r="NU25" s="6"/>
+      <c r="NV25" s="6"/>
+      <c r="NW25" s="6"/>
     </row>
-    <row r="26" spans="1:684">
-      <c r="A26" s="12" t="s">
-        <v>25</v>
-      </c>
+    <row r="26" spans="1:714">
+      <c r="A26" s="2"/>
       <c r="B26" s="4"/>
-      <c r="C26" s="12"/>
+      <c r="C26" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="D26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="NX26" s="7"/>
+      <c r="NY26" s="7"/>
+      <c r="NZ26" s="7"/>
+      <c r="OA26" s="7"/>
+      <c r="OB26" s="7"/>
+      <c r="OC26" s="7"/>
+      <c r="OD26" s="7"/>
+      <c r="OE26" s="7"/>
+      <c r="OF26" s="7"/>
+      <c r="OG26" s="7"/>
+      <c r="OH26" s="7"/>
+      <c r="OI26" s="7"/>
+      <c r="OJ26" s="7"/>
+      <c r="OK26" s="7"/>
+      <c r="OL26" s="7"/>
+      <c r="OM26" s="7"/>
+      <c r="ON26" s="7"/>
+      <c r="OO26" s="7"/>
+      <c r="OP26" s="7"/>
+      <c r="OQ26" s="7"/>
+      <c r="OR26" s="7"/>
+      <c r="OS26" s="7"/>
+      <c r="OT26" s="7"/>
+      <c r="OU26" s="7"/>
+      <c r="OV26" s="7"/>
+      <c r="OW26" s="7"/>
+      <c r="OX26" s="7"/>
+      <c r="OY26" s="7"/>
+      <c r="OZ26" s="7"/>
+      <c r="PA26" s="7"/>
+      <c r="PB26" s="7"/>
+      <c r="PC26" s="7"/>
+      <c r="PD26" s="7"/>
+      <c r="PE26" s="7"/>
+      <c r="PF26" s="7"/>
+      <c r="PG26" s="7"/>
+      <c r="PH26" s="7"/>
+      <c r="PI26" s="7"/>
+      <c r="PJ26" s="7"/>
+      <c r="PK26" s="7"/>
+      <c r="PL26" s="7"/>
+      <c r="PM26" s="7"/>
+      <c r="PN26" s="7"/>
+      <c r="PO26" s="7"/>
+      <c r="PP26" s="7"/>
+      <c r="PQ26" s="7"/>
+      <c r="PR26" s="7"/>
+      <c r="PS26" s="7"/>
+      <c r="PT26" s="7"/>
+      <c r="PU26" s="7"/>
+      <c r="PV26" s="7"/>
+      <c r="PW26" s="7"/>
+      <c r="PX26" s="7"/>
+      <c r="PY26" s="7"/>
+      <c r="PZ26" s="7"/>
+      <c r="QA26" s="7"/>
+      <c r="QB26" s="7"/>
+      <c r="QC26" s="7"/>
+      <c r="QD26" s="7"/>
+      <c r="QE26" s="7"/>
+      <c r="QF26" s="7"/>
+      <c r="QG26" s="7"/>
+      <c r="QH26" s="7"/>
+      <c r="QI26" s="7"/>
+      <c r="QJ26" s="7"/>
+      <c r="QK26" s="7"/>
+      <c r="QL26" s="7"/>
+      <c r="QM26" s="7"/>
+      <c r="QN26" s="7"/>
+      <c r="QO26" s="7"/>
+      <c r="QP26" s="7"/>
+      <c r="QQ26" s="7"/>
+      <c r="QR26" s="7"/>
+      <c r="QS26" s="7"/>
+      <c r="QT26" s="7"/>
+      <c r="QU26" s="7"/>
+      <c r="QV26" s="7"/>
+      <c r="QW26" s="7"/>
+      <c r="QX26" s="7"/>
+      <c r="QY26" s="7"/>
+    </row>
+    <row r="27" spans="1:714">
+      <c r="A27" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="NP26" s="13"/>
-      <c r="NQ26" s="13"/>
-      <c r="NR26" s="13"/>
-      <c r="NS26" s="13"/>
-      <c r="NT26" s="13"/>
-      <c r="NU26" s="13"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="QZ27" s="12"/>
+      <c r="RA27" s="12"/>
+      <c r="RB27" s="12"/>
+      <c r="RC27" s="12"/>
+      <c r="RD27" s="12"/>
+      <c r="RE27" s="12"/>
+      <c r="RF27" s="12"/>
+      <c r="RG27" s="12"/>
+      <c r="RH27" s="12"/>
+      <c r="RI27" s="12"/>
+      <c r="RJ27" s="12"/>
+      <c r="RK27" s="12"/>
+      <c r="RL27" s="12"/>
+      <c r="RM27" s="12"/>
+      <c r="RN27" s="12"/>
+      <c r="RO27" s="12"/>
+      <c r="RP27" s="12"/>
+      <c r="RQ27" s="12"/>
+      <c r="RR27" s="12"/>
+      <c r="RS27" s="12"/>
+      <c r="RT27" s="12"/>
+      <c r="RU27" s="12"/>
+      <c r="RV27" s="12"/>
+      <c r="RW27" s="12"/>
+      <c r="RX27" s="12"/>
+      <c r="RY27" s="12"/>
+      <c r="RZ27" s="12"/>
+      <c r="SA27" s="12"/>
+      <c r="SB27" s="12"/>
+      <c r="SC27" s="12"/>
+      <c r="SD27" s="12"/>
+      <c r="SE27" s="12"/>
+      <c r="SF27" s="12"/>
+      <c r="SG27" s="12"/>
+      <c r="SH27" s="12"/>
+      <c r="SI27" s="12"/>
+      <c r="SJ27" s="12"/>
+      <c r="SK27" s="12"/>
+      <c r="SL27" s="12"/>
+      <c r="SM27" s="12"/>
+      <c r="SN27" s="12"/>
+      <c r="SO27" s="12"/>
+      <c r="SP27" s="12"/>
+      <c r="SQ27" s="12"/>
+      <c r="SR27" s="12"/>
+      <c r="SS27" s="12"/>
+      <c r="ST27" s="12"/>
+      <c r="SU27" s="12"/>
+      <c r="SV27" s="12"/>
+      <c r="SW27" s="12"/>
+      <c r="SX27" s="12"/>
+      <c r="SY27" s="12"/>
+      <c r="SZ27" s="12"/>
+      <c r="TA27" s="12"/>
+      <c r="TB27" s="12"/>
+      <c r="TC27" s="12"/>
+      <c r="TD27" s="12"/>
+      <c r="TE27" s="12"/>
+      <c r="TF27" s="12"/>
+      <c r="TG27" s="12"/>
+      <c r="TH27" s="12"/>
+      <c r="TI27" s="12"/>
+      <c r="TJ27" s="12"/>
+      <c r="TK27" s="12"/>
+      <c r="TL27" s="12"/>
+      <c r="TM27" s="12"/>
+      <c r="TN27" s="12"/>
+      <c r="TO27" s="12"/>
     </row>
-    <row r="27" spans="1:684">
-      <c r="A27" s="2"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="NV27" s="7"/>
-      <c r="NW27" s="7"/>
-      <c r="NX27" s="7"/>
-      <c r="NY27" s="7"/>
-      <c r="NZ27" s="7"/>
-      <c r="OA27" s="7"/>
-      <c r="OB27" s="7"/>
-      <c r="OC27" s="7"/>
-      <c r="OD27" s="7"/>
-      <c r="OE27" s="7"/>
-      <c r="OF27" s="7"/>
-      <c r="OG27" s="7"/>
-      <c r="OH27" s="7"/>
-      <c r="OI27" s="7"/>
-      <c r="OJ27" s="7"/>
-      <c r="OK27" s="7"/>
-      <c r="OL27" s="7"/>
-      <c r="OM27" s="7"/>
-      <c r="ON27" s="7"/>
-      <c r="OO27" s="7"/>
-      <c r="OP27" s="7"/>
-      <c r="OQ27" s="7"/>
-      <c r="OR27" s="7"/>
-      <c r="OS27" s="7"/>
-      <c r="OT27" s="7"/>
-      <c r="OU27" s="7"/>
-      <c r="OV27" s="7"/>
-      <c r="OW27" s="7"/>
-      <c r="OX27" s="7"/>
-      <c r="OY27" s="7"/>
-      <c r="OZ27" s="7"/>
-      <c r="PA27" s="7"/>
-      <c r="PB27" s="7"/>
-      <c r="PC27" s="7"/>
-      <c r="PD27" s="7"/>
-      <c r="PE27" s="7"/>
-      <c r="PF27" s="7"/>
-      <c r="PG27" s="7"/>
-      <c r="PH27" s="7"/>
-      <c r="PI27" s="7"/>
-      <c r="PJ27" s="7"/>
-      <c r="PK27" s="7"/>
-      <c r="PL27" s="7"/>
-      <c r="PM27" s="7"/>
-      <c r="PN27" s="7"/>
-      <c r="PO27" s="7"/>
-      <c r="PP27" s="7"/>
-      <c r="PQ27" s="7"/>
-      <c r="PR27" s="7"/>
-      <c r="PS27" s="7"/>
-      <c r="PT27" s="7"/>
-      <c r="PU27" s="7"/>
-      <c r="PV27" s="7"/>
-      <c r="PW27" s="7"/>
-      <c r="PX27" s="7"/>
-      <c r="PY27" s="7"/>
-      <c r="PZ27" s="7"/>
-      <c r="QA27" s="7"/>
-      <c r="QB27" s="7"/>
-      <c r="QC27" s="7"/>
-      <c r="QD27" s="7"/>
-      <c r="QE27" s="7"/>
-      <c r="QF27" s="7"/>
-      <c r="QG27" s="7"/>
-      <c r="QH27" s="7"/>
-      <c r="QI27" s="7"/>
-      <c r="QJ27" s="7"/>
-      <c r="QK27" s="7"/>
-      <c r="QL27" s="7"/>
-      <c r="QM27" s="7"/>
-      <c r="QN27" s="7"/>
-      <c r="QO27" s="7"/>
-      <c r="QP27" s="7"/>
-      <c r="QQ27" s="7"/>
-      <c r="QR27" s="7"/>
-      <c r="QS27" s="7"/>
-      <c r="QT27" s="7"/>
-      <c r="QU27" s="7"/>
-      <c r="QV27" s="7"/>
-      <c r="QW27" s="7"/>
+    <row r="28" spans="1:714">
+      <c r="A28" s="2"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="TO28" s="7"/>
+      <c r="TP28" s="7"/>
+      <c r="TQ28" s="7"/>
+      <c r="TR28" s="7"/>
+      <c r="TS28" s="7"/>
+      <c r="TT28" s="7"/>
+      <c r="TU28" s="7"/>
+      <c r="TV28" s="7"/>
+      <c r="TW28" s="7"/>
+      <c r="TX28" s="7"/>
+      <c r="TY28" s="7"/>
+      <c r="TZ28" s="7"/>
+      <c r="UA28" s="7"/>
+      <c r="UB28" s="7"/>
+      <c r="UC28" s="7"/>
+      <c r="UD28" s="7"/>
+      <c r="UE28" s="7"/>
+      <c r="UF28" s="7"/>
+      <c r="UG28" s="7"/>
+      <c r="UH28" s="7"/>
+      <c r="UI28" s="7"/>
+      <c r="UJ28" s="7"/>
+      <c r="UK28" s="7"/>
+      <c r="UL28" s="7"/>
+      <c r="UM28" s="7"/>
+      <c r="UN28" s="7"/>
+      <c r="UO28" s="7"/>
+      <c r="UP28" s="7"/>
+      <c r="UQ28" s="7"/>
+      <c r="UR28" s="7"/>
+      <c r="US28" s="7"/>
+      <c r="UT28" s="7"/>
+      <c r="UU28" s="7"/>
+      <c r="UV28" s="7"/>
+      <c r="UW28" s="7"/>
+      <c r="UX28" s="7"/>
+      <c r="UY28" s="7"/>
+      <c r="UZ28" s="7"/>
+      <c r="VA28" s="7"/>
+      <c r="VB28" s="7"/>
+      <c r="VC28" s="7"/>
+      <c r="VD28" s="7"/>
+      <c r="VE28" s="7"/>
+      <c r="VF28" s="7"/>
+      <c r="VG28" s="7"/>
+      <c r="VH28" s="7"/>
+      <c r="VI28" s="7"/>
+      <c r="VJ28" s="7"/>
+      <c r="VK28" s="7"/>
+      <c r="VL28" s="7"/>
+      <c r="VM28" s="7"/>
+      <c r="VN28" s="7"/>
+      <c r="VO28" s="7"/>
+      <c r="VP28" s="7"/>
+      <c r="VQ28" s="7"/>
+      <c r="VR28" s="7"/>
+      <c r="VS28" s="7"/>
+      <c r="VT28" s="7"/>
+      <c r="VU28" s="7"/>
+      <c r="VV28" s="7"/>
+      <c r="VW28" s="7"/>
+      <c r="VX28" s="7"/>
+      <c r="VY28" s="7"/>
+      <c r="VZ28" s="7"/>
+      <c r="WA28" s="7"/>
+      <c r="WB28" s="7"/>
+      <c r="WC28" s="7"/>
+      <c r="WD28" s="7"/>
+      <c r="WE28" s="7"/>
+      <c r="WF28" s="7"/>
+      <c r="WG28" s="7"/>
     </row>
-    <row r="28" spans="1:684">
-      <c r="A28" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="QX28" s="13"/>
-      <c r="QY28" s="13"/>
-      <c r="QZ28" s="13"/>
-      <c r="RA28" s="13"/>
-      <c r="RB28" s="13"/>
-      <c r="RC28" s="13"/>
-      <c r="RD28" s="13"/>
-      <c r="RE28" s="13"/>
-      <c r="RF28" s="13"/>
-      <c r="RG28" s="13"/>
-      <c r="RH28" s="13"/>
-      <c r="RI28" s="13"/>
-      <c r="RJ28" s="13"/>
-      <c r="RK28" s="13"/>
-      <c r="RL28" s="13"/>
-      <c r="RM28" s="13"/>
-      <c r="RN28" s="13"/>
-      <c r="RO28" s="13"/>
-      <c r="RP28" s="13"/>
-      <c r="RQ28" s="13"/>
-      <c r="RR28" s="13"/>
-      <c r="RS28" s="13"/>
-      <c r="RT28" s="13"/>
-      <c r="RU28" s="13"/>
-      <c r="RV28" s="13"/>
-      <c r="RW28" s="13"/>
-      <c r="RX28" s="13"/>
-      <c r="RY28" s="13"/>
-      <c r="RZ28" s="13"/>
-      <c r="SA28" s="13"/>
-      <c r="SB28" s="13"/>
-      <c r="SC28" s="13"/>
-      <c r="SD28" s="13"/>
-      <c r="SE28" s="13"/>
-      <c r="SF28" s="13"/>
-      <c r="SG28" s="13"/>
-      <c r="SH28" s="13"/>
-      <c r="SI28" s="13"/>
-      <c r="SJ28" s="13"/>
-      <c r="SK28" s="13"/>
-      <c r="SL28" s="13"/>
-      <c r="SM28" s="13"/>
-      <c r="SN28" s="13"/>
-      <c r="SO28" s="13"/>
-      <c r="SP28" s="13"/>
-      <c r="SQ28" s="13"/>
-      <c r="SR28" s="13"/>
-      <c r="SS28" s="13"/>
-      <c r="ST28" s="13"/>
-      <c r="SU28" s="13"/>
-      <c r="SV28" s="13"/>
-      <c r="SW28" s="13"/>
-      <c r="SX28" s="13"/>
-      <c r="SY28" s="13"/>
-      <c r="SZ28" s="13"/>
-      <c r="TA28" s="13"/>
-      <c r="TB28" s="13"/>
-      <c r="TC28" s="13"/>
-      <c r="TD28" s="13"/>
-      <c r="TE28" s="13"/>
-      <c r="TF28" s="13"/>
-      <c r="TG28" s="13"/>
-      <c r="TH28" s="13"/>
-      <c r="TI28" s="13"/>
-      <c r="TJ28" s="13"/>
-      <c r="TK28" s="13"/>
-      <c r="TL28" s="13"/>
-      <c r="TM28" s="13"/>
-      <c r="TN28" s="13"/>
-      <c r="TO28" s="13"/>
-    </row>
-    <row r="29" spans="1:684">
+    <row r="29" spans="1:714">
       <c r="A29" s="2"/>
       <c r="B29" s="4"/>
       <c r="C29" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="TO29" s="7"/>
-      <c r="TP29" s="7"/>
-      <c r="TQ29" s="7"/>
-      <c r="TR29" s="7"/>
-      <c r="TS29" s="7"/>
-      <c r="TT29" s="7"/>
-      <c r="TU29" s="7"/>
-      <c r="TV29" s="7"/>
-      <c r="TW29" s="7"/>
-      <c r="TX29" s="7"/>
-      <c r="TY29" s="7"/>
-      <c r="TZ29" s="7"/>
-      <c r="UA29" s="7"/>
-      <c r="UB29" s="7"/>
-      <c r="UC29" s="7"/>
-      <c r="UD29" s="7"/>
-      <c r="UE29" s="7"/>
-      <c r="UF29" s="7"/>
-      <c r="UG29" s="7"/>
-      <c r="UH29" s="7"/>
-      <c r="UI29" s="7"/>
-      <c r="UJ29" s="7"/>
-      <c r="UK29" s="7"/>
-      <c r="UL29" s="7"/>
-      <c r="UM29" s="7"/>
-      <c r="UN29" s="7"/>
-      <c r="UO29" s="7"/>
-      <c r="UP29" s="7"/>
-      <c r="UQ29" s="7"/>
-      <c r="UR29" s="7"/>
-      <c r="US29" s="7"/>
-      <c r="UT29" s="7"/>
-      <c r="UU29" s="7"/>
-      <c r="UV29" s="7"/>
-      <c r="UW29" s="7"/>
-      <c r="UX29" s="7"/>
-      <c r="UY29" s="7"/>
-      <c r="UZ29" s="7"/>
-      <c r="VA29" s="7"/>
-      <c r="VB29" s="7"/>
-      <c r="VC29" s="7"/>
-      <c r="VD29" s="7"/>
-      <c r="VE29" s="7"/>
-      <c r="VF29" s="7"/>
-      <c r="VG29" s="7"/>
-      <c r="VH29" s="7"/>
-      <c r="VI29" s="7"/>
-      <c r="VJ29" s="7"/>
-      <c r="VK29" s="7"/>
-      <c r="VL29" s="7"/>
-      <c r="VM29" s="7"/>
-      <c r="VN29" s="7"/>
-      <c r="VO29" s="7"/>
-      <c r="VP29" s="7"/>
-      <c r="VQ29" s="7"/>
-      <c r="VR29" s="7"/>
-      <c r="VS29" s="7"/>
-      <c r="VT29" s="7"/>
-      <c r="VU29" s="7"/>
-      <c r="VV29" s="7"/>
-      <c r="VW29" s="7"/>
-      <c r="VX29" s="7"/>
-      <c r="VY29" s="7"/>
-      <c r="VZ29" s="7"/>
-      <c r="WA29" s="7"/>
-      <c r="WB29" s="7"/>
-      <c r="WC29" s="7"/>
-      <c r="WD29" s="7"/>
-      <c r="WE29" s="7"/>
-      <c r="WF29" s="7"/>
-      <c r="WG29" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="WG29" s="8"/>
+      <c r="WH29" s="8"/>
+      <c r="WI29" s="8"/>
+      <c r="WJ29" s="8"/>
+      <c r="WK29" s="8"/>
+      <c r="WL29" s="8"/>
+      <c r="WM29" s="8"/>
+      <c r="WN29" s="8"/>
+      <c r="WO29" s="8"/>
+      <c r="WP29" s="8"/>
+      <c r="WQ29" s="8"/>
+      <c r="WR29" s="8"/>
+      <c r="WS29" s="8"/>
+      <c r="WT29" s="8"/>
+      <c r="WU29" s="8"/>
+      <c r="WV29" s="8"/>
+      <c r="WW29" s="8"/>
+      <c r="WX29" s="8"/>
+      <c r="WY29" s="8"/>
+      <c r="WZ29" s="8"/>
+      <c r="XA29" s="8"/>
+      <c r="XB29" s="8"/>
+      <c r="XC29" s="8"/>
+      <c r="XD29" s="8"/>
+      <c r="XE29" s="8"/>
+      <c r="XF29" s="8"/>
+      <c r="XG29" s="8"/>
+      <c r="XH29" s="8"/>
+      <c r="XI29" s="8"/>
+      <c r="XJ29" s="8"/>
     </row>
-    <row r="30" spans="1:684">
+    <row r="30" spans="1:714">
       <c r="A30" s="2"/>
       <c r="B30" s="4"/>
       <c r="C30" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="WG30" s="8"/>
-      <c r="WH30" s="8"/>
-      <c r="WI30" s="8"/>
-      <c r="WJ30" s="8"/>
-      <c r="WK30" s="8"/>
-      <c r="WL30" s="8"/>
-      <c r="WM30" s="8"/>
-      <c r="WN30" s="8"/>
-      <c r="WO30" s="8"/>
-      <c r="WP30" s="8"/>
-      <c r="WQ30" s="8"/>
-      <c r="WR30" s="8"/>
-      <c r="WS30" s="8"/>
-      <c r="WT30" s="8"/>
-      <c r="WU30" s="8"/>
-      <c r="WV30" s="8"/>
-      <c r="WW30" s="8"/>
-      <c r="WX30" s="8"/>
-      <c r="WY30" s="8"/>
-      <c r="WZ30" s="8"/>
-      <c r="XA30" s="8"/>
-      <c r="XB30" s="8"/>
-      <c r="XC30" s="8"/>
-      <c r="XD30" s="8"/>
-      <c r="XE30" s="8"/>
-      <c r="XF30" s="8"/>
-      <c r="XG30" s="8"/>
-      <c r="XH30" s="8"/>
-      <c r="XI30" s="8"/>
-      <c r="XJ30" s="8"/>
+        <v>17</v>
+      </c>
+      <c r="XK30" s="9"/>
+      <c r="XL30" s="9"/>
+      <c r="XM30" s="9"/>
+      <c r="XN30" s="9"/>
+      <c r="XO30" s="9"/>
+      <c r="XP30" s="9"/>
+      <c r="XQ30" s="9"/>
+      <c r="XR30" s="9"/>
+      <c r="XS30" s="9"/>
+      <c r="XT30" s="9"/>
+      <c r="XU30" s="9"/>
+      <c r="XV30" s="9"/>
+      <c r="XW30" s="9"/>
+      <c r="XX30" s="9"/>
+      <c r="XY30" s="9"/>
+      <c r="XZ30" s="9"/>
+      <c r="YA30" s="9"/>
+      <c r="YB30" s="9"/>
+      <c r="YC30" s="9"/>
+      <c r="YD30" s="9"/>
+      <c r="YE30" s="9"/>
+      <c r="YF30" s="9"/>
+      <c r="YG30" s="9"/>
+      <c r="YH30" s="9"/>
+      <c r="YI30" s="9"/>
+      <c r="YJ30" s="9"/>
+      <c r="YK30" s="9"/>
+      <c r="YL30" s="9"/>
+      <c r="YM30" s="9"/>
+      <c r="YN30" s="9"/>
     </row>
-    <row r="31" spans="1:684">
+    <row r="31" spans="1:714">
       <c r="A31" s="2"/>
       <c r="B31" s="4"/>
       <c r="C31" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="XK31" s="9"/>
-      <c r="XL31" s="9"/>
-      <c r="XM31" s="9"/>
-      <c r="XN31" s="9"/>
-      <c r="XO31" s="9"/>
-      <c r="XP31" s="9"/>
-      <c r="XQ31" s="9"/>
-      <c r="XR31" s="9"/>
-      <c r="XS31" s="9"/>
-      <c r="XT31" s="9"/>
-      <c r="XU31" s="9"/>
-      <c r="XV31" s="9"/>
-      <c r="XW31" s="9"/>
-      <c r="XX31" s="9"/>
-      <c r="XY31" s="9"/>
-      <c r="XZ31" s="9"/>
-      <c r="YA31" s="9"/>
-      <c r="YB31" s="9"/>
-      <c r="YC31" s="9"/>
-      <c r="YD31" s="9"/>
-      <c r="YE31" s="9"/>
-      <c r="YF31" s="9"/>
-      <c r="YG31" s="9"/>
-      <c r="YH31" s="9"/>
-      <c r="YI31" s="9"/>
-      <c r="YJ31" s="9"/>
-      <c r="YK31" s="9"/>
-      <c r="YL31" s="9"/>
-      <c r="YM31" s="9"/>
-      <c r="YN31" s="9"/>
+        <v>19</v>
+      </c>
+      <c r="YO31" s="5"/>
+      <c r="YP31" s="5"/>
+      <c r="YQ31" s="5"/>
+      <c r="YR31" s="5"/>
+      <c r="YS31" s="5"/>
+      <c r="YT31" s="5"/>
+      <c r="YU31" s="5"/>
+      <c r="YV31" s="5"/>
+      <c r="YW31" s="5"/>
+      <c r="YX31" s="5"/>
+      <c r="YY31" s="5"/>
+      <c r="YZ31" s="5"/>
+      <c r="ZA31" s="5"/>
+      <c r="ZB31" s="5"/>
+      <c r="ZC31" s="5"/>
+      <c r="ZD31" s="5"/>
+      <c r="ZE31" s="5"/>
+      <c r="ZF31" s="5"/>
+      <c r="ZG31" s="5"/>
+      <c r="ZH31" s="5"/>
     </row>
-    <row r="32" spans="1:684">
+    <row r="32" spans="1:714">
       <c r="A32" s="2"/>
       <c r="B32" s="4"/>
       <c r="C32" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="YO32" s="10"/>
-      <c r="YP32" s="10"/>
-      <c r="YQ32" s="10"/>
-      <c r="YR32" s="10"/>
-      <c r="YS32" s="10"/>
-      <c r="YT32" s="10"/>
-      <c r="YU32" s="10"/>
-      <c r="YV32" s="10"/>
-      <c r="YW32" s="10"/>
-      <c r="YX32" s="10"/>
-      <c r="YY32" s="10"/>
-      <c r="YZ32" s="10"/>
-      <c r="ZA32" s="10"/>
-      <c r="ZB32" s="10"/>
-      <c r="ZC32" s="10"/>
-      <c r="ZD32" s="10"/>
-      <c r="ZE32" s="10"/>
-      <c r="ZF32" s="10"/>
-      <c r="ZG32" s="10"/>
-      <c r="ZH32" s="10"/>
+        <v>17</v>
+      </c>
+      <c r="ZI32" s="10"/>
+      <c r="ZJ32" s="10"/>
+      <c r="ZK32" s="10"/>
+      <c r="ZL32" s="10"/>
+      <c r="ZM32" s="10"/>
+      <c r="ZN32" s="10"/>
+      <c r="ZO32" s="10"/>
+      <c r="ZP32" s="10"/>
+      <c r="ZQ32" s="10"/>
+      <c r="ZR32" s="10"/>
+      <c r="ZS32" s="10"/>
+      <c r="ZT32" s="10"/>
+      <c r="ZU32" s="10"/>
+      <c r="ZV32" s="10"/>
+      <c r="ZW32" s="10"/>
+      <c r="ZX32" s="10"/>
+      <c r="ZY32" s="10"/>
+      <c r="ZZ32" s="10"/>
+      <c r="AAA32" s="10"/>
+      <c r="AAB32" s="10"/>
+      <c r="AAC32" s="10"/>
+      <c r="AAD32" s="10"/>
+      <c r="AAE32" s="10"/>
+      <c r="AAF32" s="10"/>
+      <c r="AAG32" s="10"/>
+      <c r="AAH32" s="10"/>
+      <c r="AAI32" s="10"/>
+      <c r="AAJ32" s="10"/>
+      <c r="AAK32" s="10"/>
+      <c r="AAL32" s="10"/>
     </row>
-    <row r="33" spans="1:864">
-      <c r="A33" s="2"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="ZI33" s="11"/>
-      <c r="ZJ33" s="11"/>
-      <c r="ZK33" s="11"/>
-      <c r="ZL33" s="11"/>
-      <c r="ZM33" s="11"/>
-      <c r="ZN33" s="11"/>
-      <c r="ZO33" s="11"/>
-      <c r="ZP33" s="11"/>
-      <c r="ZQ33" s="11"/>
-      <c r="ZR33" s="11"/>
-      <c r="ZS33" s="11"/>
-      <c r="ZT33" s="11"/>
-      <c r="ZU33" s="11"/>
-      <c r="ZV33" s="11"/>
-      <c r="ZW33" s="11"/>
-      <c r="ZX33" s="11"/>
-      <c r="ZY33" s="11"/>
-      <c r="ZZ33" s="11"/>
-      <c r="AAA33" s="11"/>
-      <c r="AAB33" s="11"/>
-      <c r="AAC33" s="11"/>
-      <c r="AAD33" s="11"/>
-      <c r="AAE33" s="11"/>
-      <c r="AAF33" s="11"/>
-      <c r="AAG33" s="11"/>
-      <c r="AAH33" s="11"/>
-      <c r="AAI33" s="11"/>
-      <c r="AAJ33" s="11"/>
-      <c r="AAK33" s="11"/>
-      <c r="AAL33" s="11"/>
+    <row r="34" spans="1:864">
+      <c r="A34" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="3">
+        <v>4</v>
+      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+      <c r="P34" s="12"/>
+      <c r="Q34" s="12"/>
+      <c r="R34" s="12"/>
+      <c r="S34" s="12"/>
+      <c r="T34" s="12"/>
+      <c r="U34" s="12"/>
+      <c r="V34" s="12"/>
+      <c r="W34" s="12"/>
+      <c r="X34" s="12"/>
+      <c r="Y34" s="12"/>
+      <c r="Z34" s="12"/>
+      <c r="AA34" s="12"/>
+      <c r="AB34" s="12"/>
+      <c r="AC34" s="12"/>
+      <c r="AD34" s="12"/>
+      <c r="AE34" s="12"/>
+      <c r="AF34" s="12"/>
+      <c r="AG34" s="12"/>
+      <c r="AH34" s="12"/>
+      <c r="AI34" s="12"/>
+      <c r="AJ34" s="12"/>
+      <c r="AK34" s="12"/>
+      <c r="AL34" s="12"/>
+      <c r="AM34" s="12"/>
+      <c r="AN34" s="12"/>
+      <c r="AO34" s="12"/>
+      <c r="AP34" s="12"/>
+      <c r="AQ34" s="12"/>
+      <c r="AR34" s="12"/>
+      <c r="AS34" s="12"/>
+      <c r="AT34" s="12"/>
+      <c r="AU34" s="12"/>
+      <c r="AV34" s="12"/>
+      <c r="AW34" s="12"/>
+      <c r="AX34" s="12"/>
+      <c r="AY34" s="12"/>
+      <c r="AZ34" s="12"/>
+      <c r="BA34" s="12"/>
+      <c r="BB34" s="12"/>
+      <c r="BC34" s="12"/>
+      <c r="BD34" s="12"/>
+      <c r="BE34" s="12"/>
+      <c r="BF34" s="12"/>
+      <c r="BG34" s="12"/>
+      <c r="BH34" s="12"/>
+      <c r="BI34" s="12"/>
+      <c r="BJ34" s="12"/>
+      <c r="BK34" s="12"/>
+      <c r="BL34" s="12"/>
+      <c r="BM34" s="12"/>
+      <c r="BN34" s="12"/>
+      <c r="BO34" s="12"/>
+      <c r="BP34" s="12"/>
+      <c r="BQ34" s="12"/>
+      <c r="BR34" s="12"/>
+      <c r="BS34" s="12"/>
+      <c r="BT34" s="12"/>
+      <c r="BU34" s="12"/>
+      <c r="BV34" s="12"/>
+      <c r="BW34" s="12"/>
+      <c r="BX34" s="12"/>
+      <c r="BY34" s="12"/>
+      <c r="BZ34" s="12"/>
+      <c r="CA34" s="12"/>
+      <c r="CB34" s="12"/>
+      <c r="CC34" s="12"/>
+      <c r="CD34" s="12"/>
+      <c r="CE34" s="12"/>
+      <c r="CF34" s="12"/>
+      <c r="CG34" s="12"/>
+      <c r="CH34" s="12"/>
+      <c r="CI34" s="12"/>
+      <c r="CJ34" s="12"/>
+      <c r="CK34" s="12"/>
+      <c r="CL34" s="12"/>
+      <c r="CM34" s="12"/>
+      <c r="CN34" s="12"/>
+      <c r="CO34" s="12"/>
+      <c r="CP34" s="12"/>
+      <c r="CQ34" s="12"/>
+      <c r="CR34" s="12"/>
+      <c r="CS34" s="12"/>
+      <c r="CT34" s="12"/>
+      <c r="CU34" s="12"/>
+      <c r="CV34" s="12"/>
+      <c r="CW34" s="12"/>
+      <c r="CX34" s="12"/>
+      <c r="CY34" s="12"/>
+      <c r="CZ34" s="12"/>
+      <c r="DA34" s="12"/>
+      <c r="DB34" s="12"/>
+      <c r="DC34" s="12"/>
+      <c r="DD34" s="12"/>
+      <c r="DE34" s="12"/>
+      <c r="DF34" s="12"/>
+      <c r="DG34" s="12"/>
+      <c r="DH34" s="12"/>
+      <c r="DI34" s="12"/>
+      <c r="DJ34" s="12"/>
+      <c r="DK34" s="12"/>
+      <c r="DL34" s="12"/>
+      <c r="DM34" s="12"/>
+      <c r="DN34" s="12"/>
+      <c r="DO34" s="12"/>
+      <c r="DP34" s="12"/>
+      <c r="DQ34" s="12"/>
+      <c r="DR34" s="12"/>
+      <c r="DS34" s="12"/>
+      <c r="DT34" s="12"/>
+      <c r="DU34" s="12"/>
+      <c r="DV34" s="12"/>
+      <c r="DW34" s="12"/>
+      <c r="DX34" s="12"/>
+      <c r="DY34" s="12"/>
+      <c r="DZ34" s="12"/>
+      <c r="EA34" s="12"/>
+      <c r="EB34" s="12"/>
+      <c r="EC34" s="12"/>
+      <c r="ED34" s="12"/>
+      <c r="EE34" s="12"/>
+      <c r="EF34" s="12"/>
+      <c r="EG34" s="12"/>
+      <c r="EH34" s="12"/>
+      <c r="EI34" s="12"/>
+      <c r="EJ34" s="12"/>
+      <c r="EK34" s="12"/>
+      <c r="EL34" s="12"/>
+      <c r="EM34" s="12"/>
+      <c r="EN34" s="12"/>
+      <c r="EO34" s="12"/>
+      <c r="EP34" s="12"/>
+      <c r="EQ34" s="12"/>
+      <c r="ER34" s="12"/>
+      <c r="ES34" s="12"/>
+      <c r="ET34" s="12"/>
+      <c r="EU34" s="12"/>
+      <c r="EV34" s="12"/>
+      <c r="EW34" s="12"/>
+      <c r="EX34" s="12"/>
+      <c r="EY34" s="12"/>
+      <c r="EZ34" s="12"/>
+      <c r="FA34" s="12"/>
+      <c r="FB34" s="12"/>
+      <c r="FC34" s="12"/>
+      <c r="FD34" s="12"/>
+      <c r="FE34" s="12"/>
+      <c r="FF34" s="12"/>
+      <c r="FG34" s="12"/>
+      <c r="FH34" s="12"/>
+      <c r="FI34" s="12"/>
+      <c r="FJ34" s="12"/>
+      <c r="FK34" s="12"/>
+      <c r="FL34" s="12"/>
+      <c r="FM34" s="12"/>
+      <c r="FN34" s="12"/>
+      <c r="FO34" s="12"/>
+      <c r="FP34" s="12"/>
+      <c r="FQ34" s="12"/>
+      <c r="FR34" s="12"/>
+      <c r="FS34" s="12"/>
+      <c r="FT34" s="12"/>
+      <c r="FU34" s="12"/>
+      <c r="FV34" s="12"/>
+      <c r="FW34" s="12"/>
+      <c r="FX34" s="12"/>
+      <c r="FY34" s="12"/>
+      <c r="FZ34" s="12"/>
+      <c r="GA34" s="12"/>
+      <c r="GB34" s="12"/>
+      <c r="GC34" s="12"/>
+      <c r="GD34" s="12"/>
+      <c r="GE34" s="12"/>
+      <c r="GF34" s="12"/>
+      <c r="GG34" s="12"/>
+      <c r="GH34" s="12"/>
+      <c r="GI34" s="12"/>
+      <c r="GJ34" s="12"/>
+      <c r="GK34" s="12"/>
+      <c r="GL34" s="12"/>
+      <c r="GM34" s="12"/>
+      <c r="GN34" s="12"/>
+      <c r="GO34" s="12"/>
+      <c r="GP34" s="12"/>
+      <c r="GQ34" s="12"/>
+      <c r="GR34" s="12"/>
+      <c r="GS34" s="12"/>
+      <c r="GT34" s="12"/>
+      <c r="GU34" s="12"/>
+      <c r="GV34" s="12"/>
+      <c r="GW34" s="12"/>
+      <c r="GX34" s="12"/>
+      <c r="GY34" s="12"/>
+      <c r="GZ34" s="12"/>
+      <c r="HA34" s="12"/>
+      <c r="HB34" s="12"/>
+      <c r="HC34" s="12"/>
+      <c r="HD34" s="12"/>
+      <c r="HE34" s="12"/>
+      <c r="HF34" s="12"/>
+      <c r="HG34" s="12"/>
+      <c r="HH34" s="12"/>
+      <c r="HI34" s="12"/>
+      <c r="HJ34" s="12"/>
+      <c r="HK34" s="12"/>
+      <c r="HL34" s="12"/>
+      <c r="HM34" s="12"/>
+      <c r="HN34" s="12"/>
+      <c r="HO34" s="12"/>
+      <c r="HP34" s="12"/>
+      <c r="HQ34" s="12"/>
+      <c r="HR34" s="12"/>
+      <c r="HS34" s="12"/>
+      <c r="HT34" s="12"/>
+      <c r="HU34" s="12"/>
+      <c r="HV34" s="12"/>
+      <c r="HW34" s="12"/>
+      <c r="HX34" s="12"/>
+      <c r="HY34" s="12"/>
+      <c r="HZ34" s="12"/>
+      <c r="IA34" s="12"/>
+      <c r="IB34" s="12"/>
+      <c r="IC34" s="12"/>
+      <c r="ID34" s="12"/>
+      <c r="IE34" s="12"/>
+      <c r="IF34" s="12"/>
+      <c r="IG34" s="12"/>
+      <c r="IH34" s="12"/>
+      <c r="II34" s="12"/>
+      <c r="IJ34" s="12"/>
+      <c r="IK34" s="12"/>
+      <c r="IL34" s="12"/>
+      <c r="IM34" s="12"/>
+      <c r="IN34" s="12"/>
+      <c r="IO34" s="12"/>
+      <c r="IP34" s="12"/>
+      <c r="IQ34" s="12"/>
+      <c r="IR34" s="12"/>
+      <c r="IS34" s="12"/>
+      <c r="IT34" s="12"/>
+      <c r="IU34" s="12"/>
+      <c r="IV34" s="12"/>
+      <c r="IW34" s="12"/>
+      <c r="IX34" s="12"/>
+      <c r="IY34" s="12"/>
+      <c r="IZ34" s="12"/>
+      <c r="JA34" s="12"/>
+      <c r="JB34" s="12"/>
+      <c r="JC34" s="12"/>
+      <c r="JD34" s="12"/>
+      <c r="JE34" s="12"/>
+      <c r="JF34" s="12"/>
+      <c r="JG34" s="12"/>
+      <c r="JH34" s="12"/>
+      <c r="JI34" s="12"/>
+      <c r="JJ34" s="12"/>
+      <c r="JK34" s="12"/>
+      <c r="JL34" s="12"/>
+      <c r="JM34" s="12"/>
+      <c r="JN34" s="12"/>
+      <c r="JO34" s="12"/>
+      <c r="JP34" s="12"/>
+      <c r="JQ34" s="12"/>
+      <c r="JR34" s="12"/>
+      <c r="JS34" s="12"/>
+      <c r="JT34" s="12"/>
+      <c r="JU34" s="12"/>
+      <c r="JV34" s="12"/>
+      <c r="JW34" s="12"/>
+      <c r="JX34" s="12"/>
+      <c r="JY34" s="12"/>
+      <c r="JZ34" s="12"/>
+      <c r="KA34" s="12"/>
+      <c r="KB34" s="12"/>
+      <c r="KC34" s="12"/>
+      <c r="KD34" s="12"/>
+      <c r="KE34" s="12"/>
+      <c r="KF34" s="12"/>
+      <c r="KG34" s="12"/>
+      <c r="KH34" s="12"/>
+      <c r="KI34" s="12"/>
+      <c r="KJ34" s="12"/>
+      <c r="KK34" s="12"/>
+      <c r="KL34" s="12"/>
+      <c r="KM34" s="12"/>
+      <c r="KN34" s="12"/>
+      <c r="KO34" s="12"/>
+      <c r="KP34" s="12"/>
+      <c r="KQ34" s="12"/>
+      <c r="KR34" s="12"/>
+      <c r="KS34" s="12"/>
+      <c r="KT34" s="12"/>
+      <c r="KU34" s="12"/>
+      <c r="KV34" s="12"/>
+      <c r="KW34" s="12"/>
+      <c r="KX34" s="12"/>
+      <c r="KY34" s="12"/>
+      <c r="KZ34" s="12"/>
+      <c r="LA34" s="12"/>
+      <c r="LB34" s="12"/>
+      <c r="LC34" s="12"/>
+      <c r="LD34" s="12"/>
+      <c r="LE34" s="12"/>
+      <c r="LF34" s="12"/>
+      <c r="LG34" s="12"/>
+      <c r="LH34" s="12"/>
+      <c r="LI34" s="12"/>
+      <c r="LJ34" s="12"/>
+      <c r="LK34" s="12"/>
+      <c r="LL34" s="12"/>
+      <c r="LM34" s="12"/>
+      <c r="LN34" s="12"/>
+      <c r="LO34" s="12"/>
+      <c r="LP34" s="12"/>
+      <c r="LQ34" s="12"/>
+      <c r="LR34" s="12"/>
+      <c r="LS34" s="12"/>
+      <c r="LT34" s="12"/>
+      <c r="LU34" s="12"/>
+      <c r="LV34" s="12"/>
+      <c r="LW34" s="12"/>
+      <c r="LX34" s="12"/>
+      <c r="LY34" s="12"/>
+      <c r="LZ34" s="12"/>
+      <c r="MA34" s="12"/>
+      <c r="MB34" s="12"/>
+      <c r="MC34" s="12"/>
+      <c r="MD34" s="12"/>
+      <c r="ME34" s="12"/>
+      <c r="MF34" s="12"/>
+      <c r="MG34" s="12"/>
+      <c r="MH34" s="12"/>
+      <c r="MI34" s="12"/>
+      <c r="MJ34" s="12"/>
+      <c r="MK34" s="12"/>
+      <c r="ML34" s="12"/>
+      <c r="MM34" s="12"/>
+      <c r="MN34" s="12"/>
+      <c r="MO34" s="12"/>
+      <c r="MP34" s="12"/>
+      <c r="MQ34" s="12"/>
+      <c r="MR34" s="12"/>
+      <c r="MS34" s="12"/>
+      <c r="MT34" s="12"/>
+      <c r="MU34" s="12"/>
+      <c r="MV34" s="12"/>
+      <c r="MW34" s="12"/>
+      <c r="MX34" s="12"/>
+      <c r="MY34" s="12"/>
+      <c r="MZ34" s="12"/>
+      <c r="NA34" s="12"/>
+      <c r="NB34" s="12"/>
+      <c r="NC34" s="12"/>
+      <c r="ND34" s="12"/>
+      <c r="NE34" s="12"/>
+      <c r="NF34" s="12"/>
+      <c r="NG34" s="12"/>
+      <c r="NH34" s="12"/>
+      <c r="NI34" s="12"/>
+      <c r="NJ34" s="12"/>
+      <c r="NK34" s="12"/>
+      <c r="NL34" s="12"/>
+      <c r="NM34" s="12"/>
+      <c r="NN34" s="12"/>
+      <c r="NO34" s="12"/>
+      <c r="NP34" s="12"/>
+      <c r="NQ34" s="12"/>
+      <c r="NR34" s="12"/>
+      <c r="NS34" s="12"/>
+      <c r="NT34" s="12"/>
+      <c r="NU34" s="12"/>
     </row>
     <row r="35" spans="1:864">
-      <c r="A35" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B35" s="3">
-        <v>4</v>
-      </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
+      <c r="A35" s="2"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="NV35" s="5"/>
+      <c r="NW35" s="5"/>
+      <c r="NX35" s="5"/>
+      <c r="NY35" s="5"/>
+      <c r="NZ35" s="5"/>
+      <c r="OA35" s="5"/>
+      <c r="OB35" s="5"/>
+      <c r="OC35" s="5"/>
+      <c r="OD35" s="5"/>
+      <c r="OE35" s="5"/>
+      <c r="OF35" s="5"/>
+      <c r="OG35" s="5"/>
+      <c r="OH35" s="5"/>
+      <c r="OI35" s="5"/>
+      <c r="OJ35" s="5"/>
+      <c r="OK35" s="5"/>
+      <c r="OL35" s="5"/>
+      <c r="OM35" s="5"/>
+      <c r="ON35" s="5"/>
+      <c r="OO35" s="5"/>
+      <c r="OP35" s="5"/>
+      <c r="OQ35" s="5"/>
+      <c r="OR35" s="5"/>
+      <c r="OS35" s="5"/>
+      <c r="OT35" s="5"/>
+      <c r="OU35" s="5"/>
+      <c r="OV35" s="5"/>
+      <c r="OW35" s="5"/>
+      <c r="OX35" s="5"/>
+      <c r="OY35" s="5"/>
+      <c r="OZ35" s="5"/>
+      <c r="PA35" s="5"/>
+      <c r="PB35" s="5"/>
+      <c r="PC35" s="5"/>
+      <c r="PD35" s="5"/>
+      <c r="PE35" s="5"/>
+      <c r="PF35" s="5"/>
+      <c r="PG35" s="5"/>
+      <c r="PH35" s="5"/>
+      <c r="PI35" s="5"/>
+      <c r="PJ35" s="5"/>
+      <c r="PK35" s="5"/>
+      <c r="PL35" s="5"/>
+      <c r="PM35" s="5"/>
+      <c r="PN35" s="5"/>
+      <c r="PO35" s="5"/>
+      <c r="PP35" s="5"/>
+      <c r="PQ35" s="5"/>
+      <c r="PR35" s="5"/>
+      <c r="PS35" s="5"/>
+      <c r="PT35" s="5"/>
+      <c r="PU35" s="5"/>
+      <c r="PV35" s="5"/>
+      <c r="PW35" s="5"/>
+      <c r="PX35" s="5"/>
+      <c r="PY35" s="5"/>
+      <c r="PZ35" s="5"/>
+      <c r="QA35" s="5"/>
+      <c r="QB35" s="5"/>
+      <c r="QC35" s="5"/>
+      <c r="QD35" s="5"/>
+      <c r="QE35" s="5"/>
+      <c r="QF35" s="5"/>
+      <c r="QG35" s="5"/>
+      <c r="QH35" s="5"/>
+      <c r="QI35" s="5"/>
+      <c r="QJ35" s="5"/>
+      <c r="QK35" s="5"/>
+      <c r="QL35" s="5"/>
+      <c r="QM35" s="5"/>
+      <c r="QN35" s="5"/>
+      <c r="QO35" s="5"/>
+      <c r="QP35" s="5"/>
+      <c r="QQ35" s="5"/>
+      <c r="QR35" s="5"/>
+      <c r="QS35" s="5"/>
+      <c r="QT35" s="5"/>
+      <c r="QU35" s="5"/>
+      <c r="QV35" s="5"/>
+      <c r="QW35" s="5"/>
+      <c r="QX35" s="5"/>
+      <c r="QY35" s="5"/>
+      <c r="QZ35" s="5"/>
+      <c r="RA35" s="5"/>
+      <c r="RB35" s="5"/>
+      <c r="RC35" s="5"/>
+      <c r="RD35" s="5"/>
+      <c r="RE35" s="5"/>
+      <c r="RF35" s="5"/>
+      <c r="RG35" s="5"/>
+      <c r="RH35" s="5"/>
+      <c r="RI35" s="5"/>
+      <c r="RJ35" s="5"/>
+      <c r="RK35" s="5"/>
+      <c r="RL35" s="5"/>
+      <c r="RM35" s="5"/>
+      <c r="RN35" s="5"/>
+      <c r="RO35" s="5"/>
+      <c r="RP35" s="5"/>
+      <c r="RQ35" s="5"/>
+      <c r="RR35" s="5"/>
+      <c r="RS35" s="5"/>
+      <c r="RT35" s="5"/>
+      <c r="RU35" s="5"/>
+      <c r="RV35" s="5"/>
+      <c r="RW35" s="5"/>
+      <c r="RX35" s="5"/>
+      <c r="RY35" s="5"/>
+      <c r="RZ35" s="5"/>
+      <c r="SA35" s="5"/>
+      <c r="SB35" s="5"/>
+      <c r="SC35" s="5"/>
     </row>
     <row r="36" spans="1:864">
       <c r="A36" s="2"/>
       <c r="B36" s="4"/>
       <c r="C36" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="MC36" s="5"/>
-      <c r="MD36" s="5"/>
-      <c r="ME36" s="5"/>
-      <c r="MF36" s="5"/>
-      <c r="MG36" s="5"/>
-      <c r="MH36" s="5"/>
-      <c r="MI36" s="5"/>
-      <c r="MJ36" s="5"/>
-      <c r="MK36" s="5"/>
-      <c r="ML36" s="5"/>
-      <c r="MM36" s="5"/>
-      <c r="MN36" s="5"/>
-      <c r="MO36" s="5"/>
-      <c r="MP36" s="5"/>
-      <c r="MQ36" s="5"/>
-      <c r="MR36" s="5"/>
-      <c r="MS36" s="5"/>
-      <c r="MT36" s="5"/>
-      <c r="MU36" s="5"/>
-      <c r="MV36" s="5"/>
-      <c r="MW36" s="5"/>
-      <c r="MX36" s="5"/>
-      <c r="MY36" s="5"/>
-      <c r="MZ36" s="5"/>
-      <c r="NA36" s="5"/>
-      <c r="NB36" s="5"/>
-      <c r="NC36" s="5"/>
-      <c r="ND36" s="5"/>
-      <c r="NE36" s="5"/>
-      <c r="NF36" s="5"/>
-      <c r="NG36" s="5"/>
-      <c r="NH36" s="5"/>
-      <c r="NI36" s="5"/>
-      <c r="NJ36" s="5"/>
-      <c r="NK36" s="5"/>
-      <c r="NL36" s="5"/>
-      <c r="NM36" s="5"/>
-      <c r="NN36" s="5"/>
-      <c r="NO36" s="5"/>
-      <c r="NP36" s="5"/>
-      <c r="NQ36" s="5"/>
-      <c r="NR36" s="5"/>
-      <c r="NS36" s="5"/>
-      <c r="NT36" s="5"/>
-      <c r="NU36" s="5"/>
-      <c r="NV36" s="5"/>
-      <c r="NW36" s="5"/>
-      <c r="NX36" s="5"/>
-      <c r="NY36" s="5"/>
-      <c r="NZ36" s="5"/>
-      <c r="OA36" s="5"/>
-      <c r="OB36" s="5"/>
-      <c r="OC36" s="5"/>
-      <c r="OD36" s="5"/>
-      <c r="OE36" s="5"/>
-      <c r="OF36" s="5"/>
-      <c r="OG36" s="5"/>
-      <c r="OH36" s="5"/>
-      <c r="OI36" s="5"/>
-      <c r="OJ36" s="5"/>
-      <c r="OK36" s="5"/>
-      <c r="OL36" s="5"/>
-      <c r="OM36" s="5"/>
-      <c r="ON36" s="5"/>
-      <c r="OO36" s="5"/>
-      <c r="OP36" s="5"/>
-      <c r="OQ36" s="5"/>
-      <c r="OR36" s="5"/>
-      <c r="OS36" s="5"/>
-      <c r="OT36" s="5"/>
-      <c r="OU36" s="5"/>
-      <c r="OV36" s="5"/>
-      <c r="OW36" s="5"/>
-      <c r="OX36" s="5"/>
-      <c r="OY36" s="5"/>
-      <c r="OZ36" s="5"/>
-      <c r="PA36" s="5"/>
-      <c r="PB36" s="5"/>
-      <c r="PC36" s="5"/>
-      <c r="PD36" s="5"/>
-      <c r="PE36" s="5"/>
-      <c r="PF36" s="5"/>
-      <c r="PG36" s="5"/>
-      <c r="PH36" s="5"/>
-      <c r="PI36" s="5"/>
-      <c r="PJ36" s="5"/>
-      <c r="PK36" s="5"/>
-      <c r="PL36" s="5"/>
-      <c r="PM36" s="5"/>
-      <c r="PN36" s="5"/>
-      <c r="PO36" s="5"/>
-      <c r="PP36" s="5"/>
-      <c r="PQ36" s="5"/>
-      <c r="PR36" s="5"/>
-      <c r="PS36" s="5"/>
-      <c r="PT36" s="5"/>
-      <c r="PU36" s="5"/>
-      <c r="PV36" s="5"/>
-      <c r="PW36" s="5"/>
-      <c r="PX36" s="5"/>
-      <c r="PY36" s="5"/>
-      <c r="PZ36" s="5"/>
-      <c r="QA36" s="5"/>
-      <c r="QB36" s="5"/>
-      <c r="QC36" s="5"/>
-      <c r="QD36" s="5"/>
-      <c r="QE36" s="5"/>
-      <c r="QF36" s="5"/>
-      <c r="QG36" s="5"/>
-      <c r="QH36" s="5"/>
-      <c r="QI36" s="5"/>
-      <c r="QJ36" s="5"/>
+        <v>9</v>
+      </c>
+      <c r="SD36" s="6"/>
+      <c r="SE36" s="6"/>
+      <c r="SF36" s="6"/>
+      <c r="SG36" s="6"/>
+      <c r="SH36" s="6"/>
+      <c r="SI36" s="6"/>
+      <c r="SJ36" s="6"/>
+      <c r="SK36" s="6"/>
+      <c r="SL36" s="6"/>
+      <c r="SM36" s="6"/>
+      <c r="SN36" s="6"/>
+      <c r="SO36" s="6"/>
+      <c r="SP36" s="6"/>
+      <c r="SQ36" s="6"/>
+      <c r="SR36" s="6"/>
+      <c r="SS36" s="6"/>
+      <c r="ST36" s="6"/>
+      <c r="SU36" s="6"/>
+      <c r="SV36" s="6"/>
+      <c r="SW36" s="6"/>
+      <c r="SX36" s="6"/>
+      <c r="SY36" s="6"/>
+      <c r="SZ36" s="6"/>
+      <c r="TA36" s="6"/>
+      <c r="TB36" s="6"/>
+      <c r="TC36" s="6"/>
+      <c r="TD36" s="6"/>
+      <c r="TE36" s="6"/>
+      <c r="TF36" s="6"/>
+      <c r="TG36" s="6"/>
+      <c r="TH36" s="6"/>
+      <c r="TI36" s="6"/>
+      <c r="TJ36" s="6"/>
+      <c r="TK36" s="6"/>
+      <c r="TL36" s="6"/>
+      <c r="TM36" s="6"/>
+      <c r="TN36" s="6"/>
+      <c r="TO36" s="6"/>
+      <c r="TP36" s="6"/>
+      <c r="TQ36" s="6"/>
     </row>
     <row r="37" spans="1:864">
       <c r="A37" s="2"/>
       <c r="B37" s="4"/>
       <c r="C37" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="QK37" s="6"/>
-      <c r="QL37" s="6"/>
-      <c r="QM37" s="6"/>
-      <c r="QN37" s="6"/>
-      <c r="QO37" s="6"/>
-      <c r="QP37" s="6"/>
-      <c r="QQ37" s="6"/>
-      <c r="QR37" s="6"/>
-      <c r="QS37" s="6"/>
-      <c r="QT37" s="6"/>
-      <c r="QU37" s="6"/>
-      <c r="QV37" s="6"/>
-      <c r="QW37" s="6"/>
-      <c r="QX37" s="6"/>
-      <c r="QY37" s="6"/>
-      <c r="QZ37" s="6"/>
-      <c r="RA37" s="6"/>
-      <c r="RB37" s="6"/>
-      <c r="RC37" s="6"/>
-      <c r="RD37" s="6"/>
-      <c r="RE37" s="6"/>
-      <c r="RF37" s="6"/>
-      <c r="RG37" s="6"/>
-      <c r="RH37" s="6"/>
-      <c r="RI37" s="6"/>
-      <c r="RJ37" s="6"/>
-      <c r="RK37" s="6"/>
-      <c r="RL37" s="6"/>
-      <c r="RM37" s="6"/>
-      <c r="RN37" s="6"/>
-      <c r="RO37" s="6"/>
-      <c r="RP37" s="6"/>
-      <c r="RQ37" s="6"/>
-      <c r="RR37" s="6"/>
-      <c r="RS37" s="6"/>
-      <c r="RT37" s="6"/>
-      <c r="RU37" s="6"/>
-      <c r="RV37" s="6"/>
-      <c r="RW37" s="6"/>
-      <c r="RX37" s="6"/>
+        <v>11</v>
+      </c>
+      <c r="TQ37" s="7"/>
+      <c r="TR37" s="7"/>
+      <c r="TS37" s="7"/>
+      <c r="TT37" s="7"/>
+      <c r="TU37" s="7"/>
+      <c r="TV37" s="7"/>
+      <c r="TW37" s="7"/>
+      <c r="TX37" s="7"/>
+      <c r="TY37" s="7"/>
+      <c r="TZ37" s="7"/>
+      <c r="UA37" s="7"/>
+      <c r="UB37" s="7"/>
+      <c r="UC37" s="7"/>
+      <c r="UD37" s="7"/>
+      <c r="UE37" s="7"/>
+      <c r="UF37" s="7"/>
+      <c r="UG37" s="7"/>
+      <c r="UH37" s="7"/>
+      <c r="UI37" s="7"/>
+      <c r="UJ37" s="7"/>
+      <c r="UK37" s="7"/>
+      <c r="UL37" s="7"/>
+      <c r="UM37" s="7"/>
+      <c r="UN37" s="7"/>
+      <c r="UO37" s="7"/>
+      <c r="UP37" s="7"/>
+      <c r="UQ37" s="7"/>
+      <c r="UR37" s="7"/>
+      <c r="US37" s="7"/>
+      <c r="UT37" s="7"/>
+      <c r="UU37" s="7"/>
+      <c r="UV37" s="7"/>
+      <c r="UW37" s="7"/>
+      <c r="UX37" s="7"/>
+      <c r="UY37" s="7"/>
+      <c r="UZ37" s="7"/>
+      <c r="VA37" s="7"/>
+      <c r="VB37" s="7"/>
+      <c r="VC37" s="7"/>
+      <c r="VD37" s="7"/>
+      <c r="VE37" s="7"/>
+      <c r="VF37" s="7"/>
+      <c r="VG37" s="7"/>
+      <c r="VH37" s="7"/>
+      <c r="VI37" s="7"/>
+      <c r="VJ37" s="7"/>
+      <c r="VK37" s="7"/>
+      <c r="VL37" s="7"/>
+      <c r="VM37" s="7"/>
+      <c r="VN37" s="7"/>
+      <c r="VO37" s="7"/>
+      <c r="VP37" s="7"/>
+      <c r="VQ37" s="7"/>
+      <c r="VR37" s="7"/>
+      <c r="VS37" s="7"/>
+      <c r="VT37" s="7"/>
+      <c r="VU37" s="7"/>
+      <c r="VV37" s="7"/>
+      <c r="VW37" s="7"/>
+      <c r="VX37" s="7"/>
+      <c r="VY37" s="7"/>
+      <c r="VZ37" s="7"/>
+      <c r="WA37" s="7"/>
+      <c r="WB37" s="7"/>
+      <c r="WC37" s="7"/>
+      <c r="WD37" s="7"/>
+      <c r="WE37" s="7"/>
+      <c r="WF37" s="7"/>
+      <c r="WG37" s="7"/>
+      <c r="WH37" s="7"/>
+      <c r="WI37" s="7"/>
+      <c r="WJ37" s="7"/>
+      <c r="WK37" s="7"/>
+      <c r="WL37" s="7"/>
+      <c r="WM37" s="7"/>
+      <c r="WN37" s="7"/>
+      <c r="WO37" s="7"/>
+      <c r="WP37" s="7"/>
+      <c r="WQ37" s="7"/>
+      <c r="WR37" s="7"/>
+      <c r="WS37" s="7"/>
     </row>
     <row r="38" spans="1:864">
-      <c r="A38" s="12" t="s">
-        <v>30</v>
+      <c r="A38" s="11" t="s">
+        <v>26</v>
       </c>
       <c r="B38" s="4"/>
-      <c r="C38" s="12"/>
+      <c r="C38" s="11"/>
       <c r="D38" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="RX38" s="13"/>
-      <c r="RY38" s="13"/>
-      <c r="RZ38" s="13"/>
-      <c r="SA38" s="13"/>
-      <c r="SB38" s="13"/>
-      <c r="SC38" s="13"/>
-      <c r="SD38" s="13"/>
-      <c r="SE38" s="13"/>
-      <c r="SF38" s="13"/>
-      <c r="SG38" s="13"/>
-      <c r="SH38" s="13"/>
-      <c r="SI38" s="13"/>
-      <c r="SJ38" s="13"/>
-      <c r="SK38" s="13"/>
-      <c r="SL38" s="13"/>
-      <c r="SM38" s="13"/>
-      <c r="SN38" s="13"/>
-      <c r="SO38" s="13"/>
-      <c r="SP38" s="13"/>
-      <c r="SQ38" s="13"/>
-      <c r="SR38" s="13"/>
-      <c r="SS38" s="13"/>
-      <c r="ST38" s="13"/>
-      <c r="SU38" s="13"/>
-      <c r="SV38" s="13"/>
-      <c r="SW38" s="13"/>
-      <c r="SX38" s="13"/>
-      <c r="SY38" s="13"/>
-      <c r="SZ38" s="13"/>
-      <c r="TA38" s="13"/>
-      <c r="TB38" s="13"/>
-      <c r="TC38" s="13"/>
-      <c r="TD38" s="13"/>
-      <c r="TE38" s="13"/>
-      <c r="TF38" s="13"/>
-      <c r="TG38" s="13"/>
-      <c r="TH38" s="13"/>
-      <c r="TI38" s="13"/>
-      <c r="TJ38" s="13"/>
-      <c r="TK38" s="13"/>
-      <c r="TL38" s="13"/>
-      <c r="TM38" s="13"/>
-      <c r="TN38" s="13"/>
-      <c r="TO38" s="13"/>
+        <v>27</v>
+      </c>
+      <c r="WS38" s="12"/>
+      <c r="WT38" s="12"/>
+      <c r="WU38" s="12"/>
+      <c r="WV38" s="12"/>
+      <c r="WW38" s="12"/>
+      <c r="WX38" s="12"/>
+      <c r="WY38" s="12"/>
+      <c r="WZ38" s="12"/>
+      <c r="XA38" s="12"/>
+      <c r="XB38" s="12"/>
+      <c r="XC38" s="12"/>
+      <c r="XD38" s="12"/>
+      <c r="XE38" s="12"/>
+      <c r="XF38" s="12"/>
+      <c r="XG38" s="12"/>
+      <c r="XH38" s="12"/>
+      <c r="XI38" s="12"/>
+      <c r="XJ38" s="12"/>
+      <c r="XK38" s="12"/>
+      <c r="XL38" s="12"/>
+      <c r="XM38" s="12"/>
+      <c r="XN38" s="12"/>
+      <c r="XO38" s="12"/>
+      <c r="XP38" s="12"/>
+      <c r="XQ38" s="12"/>
+      <c r="XR38" s="12"/>
+      <c r="XS38" s="12"/>
+      <c r="XT38" s="12"/>
+      <c r="XU38" s="12"/>
+      <c r="XV38" s="12"/>
+      <c r="XW38" s="12"/>
+      <c r="XX38" s="12"/>
+      <c r="XY38" s="12"/>
+      <c r="XZ38" s="12"/>
+      <c r="YA38" s="12"/>
+      <c r="YB38" s="12"/>
+      <c r="YC38" s="12"/>
+      <c r="YD38" s="12"/>
+      <c r="YE38" s="12"/>
+      <c r="YF38" s="12"/>
+      <c r="YG38" s="12"/>
+      <c r="YH38" s="12"/>
+      <c r="YI38" s="12"/>
+      <c r="YJ38" s="12"/>
+      <c r="YK38" s="12"/>
+      <c r="YL38" s="12"/>
+      <c r="YM38" s="12"/>
+      <c r="YN38" s="12"/>
+      <c r="YO38" s="12"/>
+      <c r="YP38" s="12"/>
+      <c r="YQ38" s="12"/>
+      <c r="YR38" s="12"/>
+      <c r="YS38" s="12"/>
+      <c r="YT38" s="12"/>
+      <c r="YU38" s="12"/>
+      <c r="YV38" s="12"/>
+      <c r="YW38" s="12"/>
+      <c r="YX38" s="12"/>
+      <c r="YY38" s="12"/>
+      <c r="YZ38" s="12"/>
+      <c r="ZA38" s="12"/>
+      <c r="ZB38" s="12"/>
+      <c r="ZC38" s="12"/>
+      <c r="ZD38" s="12"/>
+      <c r="ZE38" s="12"/>
+      <c r="ZF38" s="12"/>
+      <c r="ZG38" s="12"/>
+      <c r="ZH38" s="12"/>
     </row>
     <row r="39" spans="1:864">
       <c r="A39" s="2"/>
       <c r="B39" s="4"/>
       <c r="C39" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="TO39" s="7"/>
-      <c r="TP39" s="7"/>
-      <c r="TQ39" s="7"/>
-      <c r="TR39" s="7"/>
-      <c r="TS39" s="7"/>
-      <c r="TT39" s="7"/>
-      <c r="TU39" s="7"/>
-      <c r="TV39" s="7"/>
-      <c r="TW39" s="7"/>
-      <c r="TX39" s="7"/>
-      <c r="TY39" s="7"/>
-      <c r="TZ39" s="7"/>
-      <c r="UA39" s="7"/>
-      <c r="UB39" s="7"/>
-      <c r="UC39" s="7"/>
-      <c r="UD39" s="7"/>
-      <c r="UE39" s="7"/>
-      <c r="UF39" s="7"/>
-      <c r="UG39" s="7"/>
-      <c r="UH39" s="7"/>
-      <c r="UI39" s="7"/>
-      <c r="UJ39" s="7"/>
-      <c r="UK39" s="7"/>
-      <c r="UL39" s="7"/>
-      <c r="UM39" s="7"/>
-      <c r="UN39" s="7"/>
-      <c r="UO39" s="7"/>
-      <c r="UP39" s="7"/>
-      <c r="UQ39" s="7"/>
-      <c r="UR39" s="7"/>
-      <c r="US39" s="7"/>
-      <c r="UT39" s="7"/>
-      <c r="UU39" s="7"/>
-      <c r="UV39" s="7"/>
-      <c r="UW39" s="7"/>
-      <c r="UX39" s="7"/>
-      <c r="UY39" s="7"/>
-      <c r="UZ39" s="7"/>
-      <c r="VA39" s="7"/>
-      <c r="VB39" s="7"/>
-      <c r="VC39" s="7"/>
-      <c r="VD39" s="7"/>
-      <c r="VE39" s="7"/>
-      <c r="VF39" s="7"/>
-      <c r="VG39" s="7"/>
-      <c r="VH39" s="7"/>
-      <c r="VI39" s="7"/>
-      <c r="VJ39" s="7"/>
-      <c r="VK39" s="7"/>
-      <c r="VL39" s="7"/>
-      <c r="VM39" s="7"/>
-      <c r="VN39" s="7"/>
-      <c r="VO39" s="7"/>
-      <c r="VP39" s="7"/>
-      <c r="VQ39" s="7"/>
-      <c r="VR39" s="7"/>
-      <c r="VS39" s="7"/>
-      <c r="VT39" s="7"/>
-      <c r="VU39" s="7"/>
-      <c r="VV39" s="7"/>
-      <c r="VW39" s="7"/>
-      <c r="VX39" s="7"/>
-      <c r="VY39" s="7"/>
-      <c r="VZ39" s="7"/>
-      <c r="WA39" s="7"/>
-      <c r="WB39" s="7"/>
-      <c r="WC39" s="7"/>
-      <c r="WD39" s="7"/>
-      <c r="WE39" s="7"/>
-      <c r="WF39" s="7"/>
-      <c r="WG39" s="7"/>
-      <c r="WH39" s="7"/>
-      <c r="WI39" s="7"/>
-      <c r="WJ39" s="7"/>
-      <c r="WK39" s="7"/>
-      <c r="WL39" s="7"/>
-      <c r="WM39" s="7"/>
-      <c r="WN39" s="7"/>
-      <c r="WO39" s="7"/>
-      <c r="WP39" s="7"/>
-      <c r="WQ39" s="7"/>
+        <v>13</v>
+      </c>
+      <c r="ZI39" s="7"/>
+      <c r="ZJ39" s="7"/>
+      <c r="ZK39" s="7"/>
+      <c r="ZL39" s="7"/>
+      <c r="ZM39" s="7"/>
+      <c r="ZN39" s="7"/>
+      <c r="ZO39" s="7"/>
+      <c r="ZP39" s="7"/>
+      <c r="ZQ39" s="7"/>
+      <c r="ZR39" s="7"/>
+      <c r="ZS39" s="7"/>
+      <c r="ZT39" s="7"/>
+      <c r="ZU39" s="7"/>
+      <c r="ZV39" s="7"/>
+      <c r="ZW39" s="7"/>
+      <c r="ZX39" s="7"/>
+      <c r="ZY39" s="7"/>
+      <c r="ZZ39" s="7"/>
+      <c r="AAA39" s="7"/>
+      <c r="AAB39" s="7"/>
+      <c r="AAC39" s="7"/>
+      <c r="AAD39" s="7"/>
+      <c r="AAE39" s="7"/>
+      <c r="AAF39" s="7"/>
+      <c r="AAG39" s="7"/>
+      <c r="AAH39" s="7"/>
+      <c r="AAI39" s="7"/>
+      <c r="AAJ39" s="7"/>
+      <c r="AAK39" s="7"/>
+      <c r="AAL39" s="7"/>
+      <c r="AAM39" s="7"/>
+      <c r="AAN39" s="7"/>
+      <c r="AAO39" s="7"/>
+      <c r="AAP39" s="7"/>
+      <c r="AAQ39" s="7"/>
+      <c r="AAR39" s="7"/>
+      <c r="AAS39" s="7"/>
+      <c r="AAT39" s="7"/>
+      <c r="AAU39" s="7"/>
+      <c r="AAV39" s="7"/>
+      <c r="AAW39" s="7"/>
+      <c r="AAX39" s="7"/>
+      <c r="AAY39" s="7"/>
+      <c r="AAZ39" s="7"/>
+      <c r="ABA39" s="7"/>
+      <c r="ABB39" s="7"/>
+      <c r="ABC39" s="7"/>
+      <c r="ABD39" s="7"/>
+      <c r="ABE39" s="7"/>
+      <c r="ABF39" s="7"/>
+      <c r="ABG39" s="7"/>
+      <c r="ABH39" s="7"/>
+      <c r="ABI39" s="7"/>
+      <c r="ABJ39" s="7"/>
+      <c r="ABK39" s="7"/>
+      <c r="ABL39" s="7"/>
+      <c r="ABM39" s="7"/>
+      <c r="ABN39" s="7"/>
+      <c r="ABO39" s="7"/>
+      <c r="ABP39" s="7"/>
+      <c r="ABQ39" s="7"/>
+      <c r="ABR39" s="7"/>
+      <c r="ABS39" s="7"/>
+      <c r="ABT39" s="7"/>
+      <c r="ABU39" s="7"/>
+      <c r="ABV39" s="7"/>
+      <c r="ABW39" s="7"/>
+      <c r="ABX39" s="7"/>
+      <c r="ABY39" s="7"/>
+      <c r="ABZ39" s="7"/>
     </row>
     <row r="40" spans="1:864">
-      <c r="A40" s="12" t="s">
-        <v>27</v>
-      </c>
+      <c r="A40" s="2"/>
       <c r="B40" s="4"/>
-      <c r="C40" s="12"/>
+      <c r="C40" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D40" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="WQ40" s="13"/>
-      <c r="WR40" s="13"/>
-      <c r="WS40" s="13"/>
-      <c r="WT40" s="13"/>
-      <c r="WU40" s="13"/>
-      <c r="WV40" s="13"/>
-      <c r="WW40" s="13"/>
-      <c r="WX40" s="13"/>
-      <c r="WY40" s="13"/>
-      <c r="WZ40" s="13"/>
-      <c r="XA40" s="13"/>
-      <c r="XB40" s="13"/>
-      <c r="XC40" s="13"/>
-      <c r="XD40" s="13"/>
-      <c r="XE40" s="13"/>
-      <c r="XF40" s="13"/>
-      <c r="XG40" s="13"/>
-      <c r="XH40" s="13"/>
-      <c r="XI40" s="13"/>
-      <c r="XJ40" s="13"/>
-      <c r="XK40" s="13"/>
-      <c r="XL40" s="13"/>
-      <c r="XM40" s="13"/>
-      <c r="XN40" s="13"/>
-      <c r="XO40" s="13"/>
-      <c r="XP40" s="13"/>
-      <c r="XQ40" s="13"/>
-      <c r="XR40" s="13"/>
-      <c r="XS40" s="13"/>
-      <c r="XT40" s="13"/>
-      <c r="XU40" s="13"/>
-      <c r="XV40" s="13"/>
-      <c r="XW40" s="13"/>
-      <c r="XX40" s="13"/>
-      <c r="XY40" s="13"/>
-      <c r="XZ40" s="13"/>
-      <c r="YA40" s="13"/>
-      <c r="YB40" s="13"/>
-      <c r="YC40" s="13"/>
-      <c r="YD40" s="13"/>
-      <c r="YE40" s="13"/>
-      <c r="YF40" s="13"/>
-      <c r="YG40" s="13"/>
-      <c r="YH40" s="13"/>
-      <c r="YI40" s="13"/>
-      <c r="YJ40" s="13"/>
-      <c r="YK40" s="13"/>
-      <c r="YL40" s="13"/>
-      <c r="YM40" s="13"/>
-      <c r="YN40" s="13"/>
-      <c r="YO40" s="13"/>
-      <c r="YP40" s="13"/>
-      <c r="YQ40" s="13"/>
-      <c r="YR40" s="13"/>
-      <c r="YS40" s="13"/>
-      <c r="YT40" s="13"/>
-      <c r="YU40" s="13"/>
-      <c r="YV40" s="13"/>
-      <c r="YW40" s="13"/>
-      <c r="YX40" s="13"/>
-      <c r="YY40" s="13"/>
-      <c r="YZ40" s="13"/>
-      <c r="ZA40" s="13"/>
-      <c r="ZB40" s="13"/>
-      <c r="ZC40" s="13"/>
-      <c r="ZD40" s="13"/>
-      <c r="ZE40" s="13"/>
-      <c r="ZF40" s="13"/>
-      <c r="ZG40" s="13"/>
-      <c r="ZH40" s="13"/>
+        <v>15</v>
+      </c>
+      <c r="ACA40" s="8"/>
+      <c r="ACB40" s="8"/>
+      <c r="ACC40" s="8"/>
+      <c r="ACD40" s="8"/>
+      <c r="ACE40" s="8"/>
+      <c r="ACF40" s="8"/>
+      <c r="ACG40" s="8"/>
+      <c r="ACH40" s="8"/>
+      <c r="ACI40" s="8"/>
+      <c r="ACJ40" s="8"/>
+      <c r="ACK40" s="8"/>
+      <c r="ACL40" s="8"/>
+      <c r="ACM40" s="8"/>
+      <c r="ACN40" s="8"/>
+      <c r="ACO40" s="8"/>
+      <c r="ACP40" s="8"/>
+      <c r="ACQ40" s="8"/>
+      <c r="ACR40" s="8"/>
+      <c r="ACS40" s="8"/>
+      <c r="ACT40" s="8"/>
+      <c r="ACU40" s="8"/>
+      <c r="ACV40" s="8"/>
+      <c r="ACW40" s="8"/>
+      <c r="ACX40" s="8"/>
+      <c r="ACY40" s="8"/>
+      <c r="ACZ40" s="8"/>
+      <c r="ADA40" s="8"/>
+      <c r="ADB40" s="8"/>
+      <c r="ADC40" s="8"/>
+      <c r="ADD40" s="8"/>
     </row>
     <row r="41" spans="1:864">
       <c r="A41" s="2"/>
       <c r="B41" s="4"/>
       <c r="C41" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="ZI41" s="7"/>
-      <c r="ZJ41" s="7"/>
-      <c r="ZK41" s="7"/>
-      <c r="ZL41" s="7"/>
-      <c r="ZM41" s="7"/>
-      <c r="ZN41" s="7"/>
-      <c r="ZO41" s="7"/>
-      <c r="ZP41" s="7"/>
-      <c r="ZQ41" s="7"/>
-      <c r="ZR41" s="7"/>
-      <c r="ZS41" s="7"/>
-      <c r="ZT41" s="7"/>
-      <c r="ZU41" s="7"/>
-      <c r="ZV41" s="7"/>
-      <c r="ZW41" s="7"/>
-      <c r="ZX41" s="7"/>
-      <c r="ZY41" s="7"/>
-      <c r="ZZ41" s="7"/>
-      <c r="AAA41" s="7"/>
-      <c r="AAB41" s="7"/>
-      <c r="AAC41" s="7"/>
-      <c r="AAD41" s="7"/>
-      <c r="AAE41" s="7"/>
-      <c r="AAF41" s="7"/>
-      <c r="AAG41" s="7"/>
-      <c r="AAH41" s="7"/>
-      <c r="AAI41" s="7"/>
-      <c r="AAJ41" s="7"/>
-      <c r="AAK41" s="7"/>
-      <c r="AAL41" s="7"/>
-      <c r="AAM41" s="7"/>
-      <c r="AAN41" s="7"/>
-      <c r="AAO41" s="7"/>
-      <c r="AAP41" s="7"/>
-      <c r="AAQ41" s="7"/>
-      <c r="AAR41" s="7"/>
-      <c r="AAS41" s="7"/>
-      <c r="AAT41" s="7"/>
-      <c r="AAU41" s="7"/>
-      <c r="AAV41" s="7"/>
-      <c r="AAW41" s="7"/>
-      <c r="AAX41" s="7"/>
-      <c r="AAY41" s="7"/>
-      <c r="AAZ41" s="7"/>
-      <c r="ABA41" s="7"/>
-      <c r="ABB41" s="7"/>
-      <c r="ABC41" s="7"/>
-      <c r="ABD41" s="7"/>
-      <c r="ABE41" s="7"/>
-      <c r="ABF41" s="7"/>
-      <c r="ABG41" s="7"/>
-      <c r="ABH41" s="7"/>
-      <c r="ABI41" s="7"/>
-      <c r="ABJ41" s="7"/>
-      <c r="ABK41" s="7"/>
-      <c r="ABL41" s="7"/>
-      <c r="ABM41" s="7"/>
-      <c r="ABN41" s="7"/>
-      <c r="ABO41" s="7"/>
-      <c r="ABP41" s="7"/>
-      <c r="ABQ41" s="7"/>
-      <c r="ABR41" s="7"/>
-      <c r="ABS41" s="7"/>
-      <c r="ABT41" s="7"/>
-      <c r="ABU41" s="7"/>
-      <c r="ABV41" s="7"/>
-      <c r="ABW41" s="7"/>
-      <c r="ABX41" s="7"/>
-      <c r="ABY41" s="7"/>
-      <c r="ABZ41" s="7"/>
+        <v>17</v>
+      </c>
+      <c r="ADD41" s="9"/>
+      <c r="ADE41" s="9"/>
+      <c r="ADF41" s="9"/>
+      <c r="ADG41" s="9"/>
+      <c r="ADH41" s="9"/>
+      <c r="ADI41" s="9"/>
+      <c r="ADJ41" s="9"/>
+      <c r="ADK41" s="9"/>
+      <c r="ADL41" s="9"/>
+      <c r="ADM41" s="9"/>
+      <c r="ADN41" s="9"/>
+      <c r="ADO41" s="9"/>
+      <c r="ADP41" s="9"/>
+      <c r="ADQ41" s="9"/>
+      <c r="ADR41" s="9"/>
+      <c r="ADS41" s="9"/>
+      <c r="ADT41" s="9"/>
+      <c r="ADU41" s="9"/>
+      <c r="ADV41" s="9"/>
+      <c r="ADW41" s="9"/>
+      <c r="ADX41" s="9"/>
+      <c r="ADY41" s="9"/>
+      <c r="ADZ41" s="9"/>
+      <c r="AEA41" s="9"/>
+      <c r="AEB41" s="9"/>
+      <c r="AEC41" s="9"/>
+      <c r="AED41" s="9"/>
+      <c r="AEE41" s="9"/>
+      <c r="AEF41" s="9"/>
+      <c r="AEG41" s="9"/>
+      <c r="AEH41" s="9"/>
     </row>
     <row r="42" spans="1:864">
       <c r="A42" s="2"/>
       <c r="B42" s="4"/>
       <c r="C42" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="ACA42" s="8"/>
-      <c r="ACB42" s="8"/>
-      <c r="ACC42" s="8"/>
-      <c r="ACD42" s="8"/>
-      <c r="ACE42" s="8"/>
-      <c r="ACF42" s="8"/>
-      <c r="ACG42" s="8"/>
-      <c r="ACH42" s="8"/>
-      <c r="ACI42" s="8"/>
-      <c r="ACJ42" s="8"/>
-      <c r="ACK42" s="8"/>
-      <c r="ACL42" s="8"/>
-      <c r="ACM42" s="8"/>
-      <c r="ACN42" s="8"/>
-      <c r="ACO42" s="8"/>
-      <c r="ACP42" s="8"/>
-      <c r="ACQ42" s="8"/>
-      <c r="ACR42" s="8"/>
-      <c r="ACS42" s="8"/>
-      <c r="ACT42" s="8"/>
-      <c r="ACU42" s="8"/>
-      <c r="ACV42" s="8"/>
-      <c r="ACW42" s="8"/>
-      <c r="ACX42" s="8"/>
-      <c r="ACY42" s="8"/>
-      <c r="ACZ42" s="8"/>
-      <c r="ADA42" s="8"/>
-      <c r="ADB42" s="8"/>
-      <c r="ADC42" s="8"/>
-      <c r="ADD42" s="8"/>
+        <v>19</v>
+      </c>
+      <c r="AEH42" s="5"/>
+      <c r="AEI42" s="5"/>
+      <c r="AEJ42" s="5"/>
+      <c r="AEK42" s="5"/>
+      <c r="AEL42" s="5"/>
+      <c r="AEM42" s="5"/>
+      <c r="AEN42" s="5"/>
+      <c r="AEO42" s="5"/>
+      <c r="AEP42" s="5"/>
+      <c r="AEQ42" s="5"/>
+      <c r="AER42" s="5"/>
+      <c r="AES42" s="5"/>
+      <c r="AET42" s="5"/>
+      <c r="AEU42" s="5"/>
+      <c r="AEV42" s="5"/>
+      <c r="AEW42" s="5"/>
+      <c r="AEX42" s="5"/>
+      <c r="AEY42" s="5"/>
+      <c r="AEZ42" s="5"/>
+      <c r="AFA42" s="5"/>
+      <c r="AFB42" s="5"/>
     </row>
     <row r="43" spans="1:864">
       <c r="A43" s="2"/>
       <c r="B43" s="4"/>
       <c r="C43" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="ADD43" s="9"/>
-      <c r="ADE43" s="9"/>
-      <c r="ADF43" s="9"/>
-      <c r="ADG43" s="9"/>
-      <c r="ADH43" s="9"/>
-      <c r="ADI43" s="9"/>
-      <c r="ADJ43" s="9"/>
-      <c r="ADK43" s="9"/>
-      <c r="ADL43" s="9"/>
-      <c r="ADM43" s="9"/>
-      <c r="ADN43" s="9"/>
-      <c r="ADO43" s="9"/>
-      <c r="ADP43" s="9"/>
-      <c r="ADQ43" s="9"/>
-      <c r="ADR43" s="9"/>
-      <c r="ADS43" s="9"/>
-      <c r="ADT43" s="9"/>
-      <c r="ADU43" s="9"/>
-      <c r="ADV43" s="9"/>
-      <c r="ADW43" s="9"/>
-      <c r="ADX43" s="9"/>
-      <c r="ADY43" s="9"/>
-      <c r="ADZ43" s="9"/>
-      <c r="AEA43" s="9"/>
-      <c r="AEB43" s="9"/>
-      <c r="AEC43" s="9"/>
-      <c r="AED43" s="9"/>
-      <c r="AEE43" s="9"/>
-      <c r="AEF43" s="9"/>
-      <c r="AEG43" s="9"/>
-      <c r="AEH43" s="9"/>
-    </row>
-    <row r="44" spans="1:864">
-      <c r="A44" s="2"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="AEH44" s="10"/>
-      <c r="AEI44" s="10"/>
-      <c r="AEJ44" s="10"/>
-      <c r="AEK44" s="10"/>
-      <c r="AEL44" s="10"/>
-      <c r="AEM44" s="10"/>
-      <c r="AEN44" s="10"/>
-      <c r="AEO44" s="10"/>
-      <c r="AEP44" s="10"/>
-      <c r="AEQ44" s="10"/>
-      <c r="AER44" s="10"/>
-      <c r="AES44" s="10"/>
-      <c r="AET44" s="10"/>
-      <c r="AEU44" s="10"/>
-      <c r="AEV44" s="10"/>
-      <c r="AEW44" s="10"/>
-      <c r="AEX44" s="10"/>
-      <c r="AEY44" s="10"/>
-      <c r="AEZ44" s="10"/>
-      <c r="AFA44" s="10"/>
-      <c r="AFB44" s="10"/>
-    </row>
-    <row r="45" spans="1:864">
-      <c r="A45" s="2"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="AFB45" s="11"/>
-      <c r="AFC45" s="11"/>
-      <c r="AFD45" s="11"/>
-      <c r="AFE45" s="11"/>
-      <c r="AFF45" s="11"/>
-      <c r="AFG45" s="11"/>
-      <c r="AFH45" s="11"/>
-      <c r="AFI45" s="11"/>
-      <c r="AFJ45" s="11"/>
-      <c r="AFK45" s="11"/>
-      <c r="AFL45" s="11"/>
-      <c r="AFM45" s="11"/>
-      <c r="AFN45" s="11"/>
-      <c r="AFO45" s="11"/>
-      <c r="AFP45" s="11"/>
-      <c r="AFQ45" s="11"/>
-      <c r="AFR45" s="11"/>
-      <c r="AFS45" s="11"/>
-      <c r="AFT45" s="11"/>
-      <c r="AFU45" s="11"/>
-      <c r="AFV45" s="11"/>
-      <c r="AFW45" s="11"/>
-      <c r="AFX45" s="11"/>
-      <c r="AFY45" s="11"/>
-      <c r="AFZ45" s="11"/>
-      <c r="AGA45" s="11"/>
-      <c r="AGB45" s="11"/>
-      <c r="AGC45" s="11"/>
-      <c r="AGD45" s="11"/>
-      <c r="AGE45" s="11"/>
-      <c r="AGF45" s="11"/>
+      <c r="AFB43" s="10"/>
+      <c r="AFC43" s="10"/>
+      <c r="AFD43" s="10"/>
+      <c r="AFE43" s="10"/>
+      <c r="AFF43" s="10"/>
+      <c r="AFG43" s="10"/>
+      <c r="AFH43" s="10"/>
+      <c r="AFI43" s="10"/>
+      <c r="AFJ43" s="10"/>
+      <c r="AFK43" s="10"/>
+      <c r="AFL43" s="10"/>
+      <c r="AFM43" s="10"/>
+      <c r="AFN43" s="10"/>
+      <c r="AFO43" s="10"/>
+      <c r="AFP43" s="10"/>
+      <c r="AFQ43" s="10"/>
+      <c r="AFR43" s="10"/>
+      <c r="AFS43" s="10"/>
+      <c r="AFT43" s="10"/>
+      <c r="AFU43" s="10"/>
+      <c r="AFV43" s="10"/>
+      <c r="AFW43" s="10"/>
+      <c r="AFX43" s="10"/>
+      <c r="AFY43" s="10"/>
+      <c r="AFZ43" s="10"/>
+      <c r="AGA43" s="10"/>
+      <c r="AGB43" s="10"/>
+      <c r="AGC43" s="10"/>
+      <c r="AGD43" s="10"/>
+      <c r="AGE43" s="10"/>
+      <c r="AGF43" s="10"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>